<commit_message>
feat: complete course content catalog
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/input/cursos.xlsx
+++ b/input/cursos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3614" uniqueCount="2406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3944" uniqueCount="2675">
   <si>
     <t>course_id</t>
   </si>
@@ -6697,6 +6697,9 @@
     <t>ciencias-biologicas</t>
   </si>
   <si>
+    <t>Pesquise biodiversidade, evolução e biotecnologia em projetos ambientais, de saúde e de conservação da vida.</t>
+  </si>
+  <si>
     <t>O curso de Bacharelado em Ciências Biológicas semipresencial, busca formar profissionais capacitados para lidar com projetos e pesquisas voltados para o meio ambiente,saúde e biotecnologia, habilitado para compreender sobre a diversidade de formas de vida e ação de processos evolutivos, estudando de forma abrangente e completa toda a vida existente no planeta. O curso oferece material didático que fomenta o aprendizado e a curiosidade para realizar pesquisas e diversas atividades extracurriculares. Com duração de 8 semestres (4 anos), o curso fornece o diploma de Bacharel em Ciências Biológicas.</t>
   </si>
   <si>
@@ -6730,6 +6733,27 @@
     <t>Estude Ciências Biológicas a distância com a mesma qualidade do presencial. Bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Amostragem de biodiversidade em campo de pesquisa</t>
+  </si>
+  <si>
+    <t>Bióloga de cerca de 27 anos, mulher de pele negra, cabelo crespo com boné, camisa de campo, atenção à bandeja de amostras.</t>
+  </si>
+  <si>
+    <t>Trilha organizada de reserva brasileira contemporânea, vegetação, mesa dobrável, céu de manhã, espaço de pesquisa, sem consultório e sem curral.</t>
+  </si>
+  <si>
+    <t>rede entomológica, bandeja de amostras, lupa de campo, caderno, frascos vazios</t>
+  </si>
+  <si>
+    <t>Separa insetos na bandeja com a lupa e anota no caderno, em pé à direita da trilha.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; jaleco hospitalar; microscópio clínico; animal ferido; cirurgia; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional da manhã. Composição quadrada 1:1, enquadramento médio-aberto, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Bióloga, mulher de pele negra, cerca de 27 anos, boné, na trilha de reserva, separando amostras na bandeja com a lupa. Objetos: rede entomológica, bandeja, lupa, caderno e frascos. Sem jaleco hospitalar, sem microscópio clínico, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>formacao-pedagogica-geografia-semipresencial-licenciatura</t>
   </si>
   <si>
@@ -6737,6 +6761,9 @@
   </si>
   <si>
     <t>formacao-pedagogica-geografia</t>
+  </si>
+  <si>
+    <t>Monte kits de aula de espaço geográfico, mapas e coordenação escolar para quem já concluiu pedagogia.</t>
   </si>
   <si>
     <t xml:space="preserve">O curso de Formação Pedagógica em Geografia da Cruzeiro do Sul Virtual está disponível no formato Semipresencial e é destinado especificamente a alunos que já possuem uma graduação em Pedagogia. Ao longo da formação, o curso terá foco em despertar questionamento crítico e reflexivo para os profissionais dessa área da educação acerca de vários temas das geografias humana e física.
@@ -6768,6 +6795,27 @@
     <t>Conquiste sua Formação Pedagógica em Geografia semipresencial na Cruzeiro do Sul Virtual e habilite-se para dar aulas de Geografia no Ensino Fundamental e Médio.</t>
   </si>
   <si>
+    <t>Montagem de sequência didática de geografia</t>
+  </si>
+  <si>
+    <t>Formadora pedagógica de cerca de 31 anos, mulher de pele morena, cabelo pixie preto, camisa listrada, atenção à mapoteca.</t>
+  </si>
+  <si>
+    <t>Sala de mapoteca escolar brasileira contemporânea, gaveteiro de mapas, mesa alta, janela, espaço de preparação, sem turma e sem globo em uso.</t>
+  </si>
+  <si>
+    <t>gaveta de mapas mudos, cartões de aula em branco, tesoura escolar, cola, caderno pedagógico</t>
+  </si>
+  <si>
+    <t>Retira um mapa mudo da gaveta e recorta cartões de aula em branco, em pé à direita da mapoteca.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; globo como ação principal; GPS de campo; giz no quadro de turma; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Formadora pedagógica, mulher de pele morena, cerca de 31 anos, cabelo pixie, camisa listrada, retirando mapa mudo da gaveta e recortando cartões em branco. Objetos: gaveta de mapas, cartões, tesoura, cola e caderno. Sem globo em uso, sem GPS, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>fonoaudiologia-semipresencial-bacharelado</t>
   </si>
   <si>
@@ -6775,6 +6823,9 @@
   </si>
   <si>
     <t>fonoaudiologia</t>
+  </si>
+  <si>
+    <t>Acompanhe práticas de voz, linguagem, audição e deglutição com foco na comunicação e na qualidade de vida.</t>
   </si>
   <si>
     <t xml:space="preserve">O curso de Fonoaudiologia Semipresencial visa fornecer conhecimentos para que o aluno adquira competências para avaliar, diagnosticar e tratar questões ligadas à fala, voz, linguagem, audição e deglutição, desenvolvendo habilidades clínicas e técnicas para auxiliar os pacientes na melhoria da comunicação e na qualidade de vida. No curso, é proporcionado um embasamento teórico abrangendo anatomia, fisiologia, psicologia, neurologia e outras disciplinas correlatas à saúde.
@@ -6811,6 +6862,27 @@
     <t>Desenvolva habilidades em Fonoaudiologia a distância EAD com flexibilidade e qualidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Exercício de articulação e voz com espelho</t>
+  </si>
+  <si>
+    <t>Fonoaudióloga de cerca de 28 anos, mulher de pele morena, cabelo cacheado curto, camisa e colete clínico, atenção ao espelho.</t>
+  </si>
+  <si>
+    <t>Sala de práticas de comunicação em clínica acessível brasileira, espelho de parede, mesa, janela, espaço digno, sem maca de fisioterapia.</t>
+  </si>
+  <si>
+    <t>espelho, diapasão, cartões de articulação sem escritos, copo d'água, caderno</t>
+  </si>
+  <si>
+    <t>Demonstra a articulação diante do espelho e anota o exercício no caderno, em pé à direita, sem aplicar exame clínico.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; diagnóstico; cura; tratamento; elásticos de reabilitação; utensílio de cozinha adaptado; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Fonoaudióloga, mulher de pele morena, cerca de 28 anos, colete clínico, demonstrando articulação no espelho e anotando no caderno. Objetos: espelho, diapasão, cartões sem escritos, copo e caderno. Sem maca, sem exame clínico, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>engenharia-mecanica-semipresencial-bacharelado</t>
   </si>
   <si>
@@ -6818,6 +6890,9 @@
   </si>
   <si>
     <t>engenharia-mecanica</t>
+  </si>
+  <si>
+    <t>Projete, fabrique e conserve máquinas e equipamentos, com operação e decisões de engenharia mecânica.</t>
   </si>
   <si>
     <t>O bacharelado de Engenharia Mecânica semipresencial da Cruzeiro do Sul Virtual, e foca em proporcionar uma formação de qualidade, robusta e que capacita profissionais para tomar decisões criteriosas e bem fundamentadas, garantindo consistência entre ações e objetivos, habilitando-os para atuar em atividades de projeto, fabricação, operação e conservação de máquinas e equipamentos. Ao longo da graduação, os estudantes são introduzidos ao método teórico-prático, sendo preparados para atuar diretamente em questões complexas e ajudar significativamente no crescimento da engenharia mecânica. Com duração de 10 semestres (5 anos), o currículo do curso oferece uma formação ampla e alinhada às necessidades do mercado atual.</t>
@@ -6853,6 +6928,27 @@
     <t>Desenvolva habilidades em Engenharia Mecânica EAD com flexibilidade e baixo custo. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Conferência de conjunto mecânico e desenho técnico</t>
+  </si>
+  <si>
+    <t>Engenheiro mecânico de cerca de 31 anos, homem de pele negra, cabelo curto, camisa e óculos de proteção na testa, atenção à caixa de engrenagens.</t>
+  </si>
+  <si>
+    <t>Oficina de protótipos mecânicos contemporânea brasileira, bancada de metal, desenho técnico na parede, janela industrial, espaço limpo, sem robô e sem painel elétrico.</t>
+  </si>
+  <si>
+    <t>caixa de engrenagens, desenho técnico sem cotas, chave combinada, parafusos, caderno</t>
+  </si>
+  <si>
+    <t>Encaixa uma engrenagem no conjunto e aperta o parafuso com a chave, em pé à direita da bancada.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; braço robótico; quadro de distribuição elétrica; holograma; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Engenheiro mecânico, homem de pele negra, cerca de 31 anos, óculos de proteção na testa, encaixando uma engrenagem e apertando o parafuso com a chave. Objetos: caixa de engrenagens, desenho sem cotas, chave, parafusos e caderno. Sem robô, sem painel elétrico, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>estudos-teoricos-psicanaliticos-e-sociais-ead-bacharelado</t>
   </si>
   <si>
@@ -6860,6 +6956,9 @@
   </si>
   <si>
     <t>estudos-teoricos-psicanaliticos-e-sociais</t>
+  </si>
+  <si>
+    <t>Estude teorias da subjetividade, desenvolvimento psíquico e leitura social em pesquisa psicanalítica.</t>
   </si>
   <si>
     <t>O curso de Estudos Teóricos Psicanalíticos e Sociais EAD da Universidade Cruzeiro do Sul Virtual, oferece uma formação completa na teoria e prática psicanalítica. Com ênfase na compreensão da subjetividade humana, o curso aborda teorias como a freudiana, desenvolvimento psicossexual, interpretação dos sonhos e psicopatologia. Ao final dos 8 semestres (4 anos), os alunos estão preparados para atuar em projetos que envolvem a pesquisa psicanalítica em diferentes âmbitos. O curso confere o título de bacharel.</t>
@@ -6894,6 +6993,30 @@
     <t>Estude Psicanálise a distância EAD com a mesma qualidade do presencial. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Leitura comparada de teoria psicanalítica e social</t>
+  </si>
+  <si>
+    <t>Pesquisadora teórica de cerca de 26 anos, mulher de pele clara, cabelo pixie loiro escuro, camisa vinho, leitura atenta.</t>
+  </si>
+  <si>
+    <t>Sala de pesquisa com mural de conceitos em branco, mesa, caixas de fotocópias, janela, sem divã, sem consultório e sem mesa de seminário.</t>
+  </si>
+  <si>
+    <t>mural de conceitos, cartões em branco, livro fechado, caixas de fotocópias, caneta</t>
+  </si>
+  <si>
+    <t>Fixa cartões em branco no mural de conceitos e consulta o livro fechado, em pé à direita.</t>
+  </si>
+  <si>
+    <t>Formato quadrado 1:1, enquadramento médio, personagem em pé à direita, região inferior esquerda livre, nenhum rosto, mão ou objeto importante na região inferior esquerda, iluminação publicitária natural suave, separação clara entre assunto e fundo.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; divã; consulta clínica; psicoterapia; jaleco; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Pesquisadora teórica, mulher de pele clara, cerca de 26 anos, cabelo pixie, camisa vinho, fixando cartões em branco no mural de conceitos. Páginas sem escritos visíveis. Objetos: mural, cartões em branco, livro fechado, caixas e caneta. Sem divã, sem consultório, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>engenharia-da-computacao-semipresencial-bacharelado</t>
   </si>
   <si>
@@ -6901,6 +7024,9 @@
   </si>
   <si>
     <t>engenharia-da-computacao</t>
+  </si>
+  <si>
+    <t>Integre eletrônica e computação no desenvolvimento, análise e operação de sistemas eletrônicos e computacionais.</t>
   </si>
   <si>
     <t>O curso de Engenharia de Computação semipresencial da Cruzeiro do Sul, forma engenheiros por meio da combinação de teoria e prática. Integrando conhecimentos de eletrônica e computação, o curso se especializa no desenvolvimento, análise e operação de sistemas eletrônicos e computacionais. A graduação une ciências exatas a conhecimentos avançados de computação, preparando profissionais completos, competentes e prontos para o mercado e para as inovações do futuro. Com duração de 10 semestres (5 anos), o curso confere o título de bacharel em Engenharia de Computação.</t>
@@ -6939,6 +7065,30 @@
     <t>Aprenda Engenharia da Computação a distância EAD com qualidade e flexibilidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Montagem de placa e teste de sistema embarcado</t>
+  </si>
+  <si>
+    <t>Engenheiro da computação de cerca de 26 anos, homem de pele morena clara, cabelo liso curto, polo e jaleco aberto, atenção à placa.</t>
+  </si>
+  <si>
+    <t>Laboratório de hardware contemporâneo brasileiro, bancada antiestática, ferramentas alinhadas, iluminação clara, sem rack de rede e sem quadro de software.</t>
+  </si>
+  <si>
+    <t>placa de circuito, ferro de solda desligado, osciloscópio, pinça, protoboard</t>
+  </si>
+  <si>
+    <t>Encaixa um componente na placa e observa o traço no osciloscópio, sentada à direita da bancada.</t>
+  </si>
+  <si>
+    <t>Formato quadrado 1:1, enquadramento médio, personagem sentada à direita, região inferior esquerda livre, nenhum rosto, mão ou objeto importante na região inferior esquerda, iluminação publicitária de laboratório, separação clara entre assunto e fundo.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; holograma; capuz de hacker; engrenagens como cena principal; quadro de distribuição; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Engenheiro da computação, homem de pele morena clara, cerca de 26 anos, polo, encaixando componente na placa e olhando o osciloscópio. Objetos: placa, ferro desligado, osciloscópio, pinça e protoboard. Sem holograma, sem capuz, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>engenharia-eletrica-semipresencial-bacharelado</t>
   </si>
   <si>
@@ -6946,6 +7096,9 @@
   </si>
   <si>
     <t>engenharia-eletrica</t>
+  </si>
+  <si>
+    <t>Monte sistemas de geração, transmissão e distribuição de energia, com projetos elétricos e medições.</t>
   </si>
   <si>
     <t>O curso de Engenharia Elétrica semipresencial, prepara engenheiros para inovar e aplicar novas tecnologias, incentivando uma abordagem reflexiva e criativa na resolução de problemas. Considerando aspectos políticos, econômicos, sociais, ambientais e culturais, o profissional é formado com uma visão ética e humanística.Além de projetar sistemas residenciais, industriais, comerciais e de processamento de sinais digitais e analógicos, essa formação capacita os alunos para elaboração de documentação técnica detalhada, oferecendo uma sólida base teórica e prática através de laboratórios modernos e equipados. O curso tem duração de 10 semestres (5 anos) e confere o título de bacharel em Engenharia Elétrica.</t>
@@ -6982,6 +7135,30 @@
     <t>Aprenda Engenharia Elétrica a distância EAD com qualidade e flexibilidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Medição em quadro de distribuição elétrica</t>
+  </si>
+  <si>
+    <t>Engenheiro eletricista de cerca de 35 anos, homem de pele clara, barba curta, camisa, protetor auricular e óculos, multímetro na mão.</t>
+  </si>
+  <si>
+    <t>Sala elétrica industrial contemporânea brasileira, quadro aberto organizado, piso limpo, iluminação industrial, sem bancada de solda e sem engrenagens.</t>
+  </si>
+  <si>
+    <t>quadro de distribuição, multímetro, alicate isolado, prancheta, luvas</t>
+  </si>
+  <si>
+    <t>Apoia as pontas do multímetro no quadro e anota a leitura na prancheta, em pé à direita.</t>
+  </si>
+  <si>
+    <t>Formato quadrado 1:1, enquadramento médio, personagem em pé à direita, região inferior esquerda livre, nenhum rosto, mão ou objeto importante na região inferior esquerda, iluminação publicitária industrial, separação clara entre assunto e fundo.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; choque; fiação precária; placa de circuito como cena principal; holograma; ambiente de luxo.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Engenheiro eletricista, homem de pele clara, cerca de 35 anos, protetor auricular e óculos, medindo o quadro com o multímetro. Objetos: quadro, multímetro, alicate isolado, prancheta e luvas. Sem placa de circuito em destaque, sem holograma, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>letras-portugues-e-espanhol-semipresencial-licenciatura</t>
   </si>
   <si>
@@ -6989,6 +7166,9 @@
   </si>
   <si>
     <t>letras-portugues-e-espanhol</t>
+  </si>
+  <si>
+    <t>Ensine português e espanhol com literatura, cultura e produção de material didático para a educação básica.</t>
   </si>
   <si>
     <t>O curso de Licenciatura em Letras - Português e Espanhol semipresencial da Cruzeiro do Sul Virtual proporciona uma formação abrangente e integrada nas áreas de língua, literatura e cultura dos idiomas português e espanhol. Os estudantes exploram tanto a linguagem oral quanto escrita, estudam obras literárias de diversas épocas e contextos culturais.Além disso, o curso inclui o estudo dos aspectos histórico-culturais da língua espanhola oral e escrita, contribuindo para a produção de material didático de excelência e oferecendo uma orientação teórico-metodológica sólida. Isso prepara os estudantes não apenas para o ensino das línguas, mas também para participar de atividades de pesquisa e promover o intercâmbio cultural entre os povos de língua portuguesa e hispânica. Com duração de 8 semestres (4 anos), a formação confere o título de licenciatura.</t>
@@ -7027,6 +7207,27 @@
     <t>Aprenda Português e Espanhol a distância EAD com flexibilidade e qualidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Aula bilíngue com cartões ilustrados de vocabulário</t>
+  </si>
+  <si>
+    <t>Professora de letras de cerca de 25 anos, mulher de pele morena, cabelo liso com franja, blusa azul e calça, mostrando um cartão.</t>
+  </si>
+  <si>
+    <t>Laboratório de idiomas contemporâneo brasileiro, cabines com fones, mesa central, janela, espaço organizado, sem bandeiras e sem carteiras em fileira.</t>
+  </si>
+  <si>
+    <t>fones, microfone de mesa, cartões ilustrados sem escritos, livros fechados, painel de áudio</t>
+  </si>
+  <si>
+    <t>Mostra um cartão ilustrado e aponta o fone na cabine, em pé à direita da mesa central.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; bandeiras; escritos em espanhol; kanji; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento aberto, personagem na região superior direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Professora de letras, mulher de pele morena, cerca de 25 anos, blusa azul, mostrando cartão ilustrado sem escritos em laboratório de idiomas com cabines. Objetos: fones, microfone de mesa, cartões, livros fechados e painel de áudio. Sem bandeiras, sem escritos estrangeiros, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>letras-portugues-e-japones-semipresencial-licenciatura</t>
   </si>
   <si>
@@ -7034,6 +7235,9 @@
   </si>
   <si>
     <t>letras-portugues-e-japones</t>
+  </si>
+  <si>
+    <t>Explore compreensão oral, pronúncia e práticas de ensino de português e japonês, com didática e metodologia.</t>
   </si>
   <si>
     <t>O curso Letras - Português e Japonês semipresencial da Cruzeiro do Sul Virtual, sendo uma licenciatura, inclui disciplinas como didática, metodologia e práticas de ensino de línguas, preparando os estudantes para atuarem de forma eficaz nas salas de aula, enriquecendo sua vivência e experiência com os idiomas.Além disso, o curso contempla o estudo detalhado dos aspectos histórico-culturais da língua japonesa, tanto oral quanto escrita, abrangendo os sistemas hiragana, katakana e kanji. Os alunos exploram textos e obras de autores clássicos e contemporâneos, proporcionando uma compreensão profunda da cultura japonesa através da literatura e outras expressões artísticas. Com 8 semestres de duração (4 anos), o curso confere o título de licenciatura.</t>
@@ -7072,6 +7276,27 @@
     <t>Estude Português e Japonês a distância EAD com a mesma qualidade do presencial. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Compreensão oral e pronúncia em aula bilíngue</t>
+  </si>
+  <si>
+    <t>Professora de cerca de 29 anos, mulher de pele clara, cabelo preto liso preso, camisa e calça, atenção à turma e à caixa de som.</t>
+  </si>
+  <si>
+    <t>Sala de aula com carteiras em U contemporânea brasileira, caixa de som, quadro apagado, janela, espaço organizado, sem bandeiras, sem caligrafia e sem decoração temática.</t>
+  </si>
+  <si>
+    <t>caixa de som, gravador portátil, microfone de mão, livros fechados, caderno de escuta</t>
+  </si>
+  <si>
+    <t>Liga a caixa de som e demonstra a pronúncia no microfone, em pé à direita, quadro apagado.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; caligrafia; pincel; tinteiro; quimono; anime; bandeiras; caracteres legíveis; cabines de áudio; fantoche; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Professora, mulher de pele clara, cerca de 29 anos, camisa, em sala com carteiras em U, ligando a caixa de som e demonstrando a pronúncia no microfone. Objetos: caixa de som, gravador, microfone de mão, livros fechados e caderno. Sem caligrafia, sem pincel, sem quimono, sem bandeiras, sem caracteres visíveis, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>design-de-experiencia-ead-tecnologo</t>
   </si>
   <si>
@@ -7079,6 +7304,9 @@
   </si>
   <si>
     <t>design-de-experiencia</t>
+  </si>
+  <si>
+    <t>Mapeie jornadas de uso, prototipagem e testes de usabilidade centrados em produtos e serviços digitais.</t>
   </si>
   <si>
     <t>O curso de Design de Experiência EAD da Cruzeiro do Sul Virtual oferece uma formação completa para profissionais interessados em criar experiências impactantes e intuitivas para usuários de produtos e serviços digitais. Com uma abordagem prática e teórica, os alunos aprendem a aplicar princípios de psicologia, design thinking e tecnologia para desenvolver interfaces e interações que atendam às necessidades e expectativas dos usuários. Ao longo de 4 semestres (2 anos), os estudantes exploram temas como pesquisa de mercado, prototipagem, usabilidade e design centrado no usuário, preparando-se para carreiras dinâmicas em um mercado digital em constante evolução. Após a conclusão do curso, os alunos recebem a titulação de tecnólogo em Design de Experiência.</t>
@@ -7115,6 +7343,27 @@
     <t>Aprimore suas habilidades em Design de Experiência EAD com qualidade e flexibilidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Mapeamento de jornada e teste de protótipo em papel</t>
+  </si>
+  <si>
+    <t>Designer de experiência de cerca de 26 anos, mulher de pele negra, cabelo black curto, camisa oversized e calça, atenção ao mural de jornada.</t>
+  </si>
+  <si>
+    <t>Sala de pesquisa de usuário contemporânea brasileira, mural, mesa com protótipos de papel, janela, espaço acessível, sem tapete de corte e sem notebook de código.</t>
+  </si>
+  <si>
+    <t>mural de jornada com cartões em branco, protótipo de papel, caneta, cronômetro, adesivos em branco</t>
+  </si>
+  <si>
+    <t>Move um cartão no mural da jornada e observa a pessoa testando o protótipo de papel, em pé à direita.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; código na tela; tesoura de diagramação; holograma; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Designer de experiência, mulher de pele negra, cerca de 26 anos, camisa oversized, movendo cartão em branco no mural de jornada. Objetos: mural, protótipo de papel, caneta, cronômetro e adesivos em branco. Sem código, sem tapete de corte, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>historia-ead-bacharelado</t>
   </si>
   <si>
@@ -7122,6 +7371,9 @@
   </si>
   <si>
     <t>historia</t>
+  </si>
+  <si>
+    <t>Analise fontes históricas e seus reflexos sociais, políticos, econômicos e culturais na sociedade atual.</t>
   </si>
   <si>
     <t>A graduação de História EAD na modalidade Bacharelado, Cruzeiro do Sul Virtual, tem duração de 6 semestres (3 anos), e capacita os estudantes para terem clareza sobre os eventos históricos e seu reflexo na sociedade atual. O curso aborda e analisa períodos históricos diversos, a fim de torná-los aptos para a pesquisa histórica e análise crítica. Com uma abordagem integrada, o curso explora aspectos sociais, políticos, religiosos, econômicos e culturais, formando uma base histórica que capacita os graduados para diversas áreas de trabalho.</t>
@@ -7157,6 +7409,30 @@
     <t>Aprofunde-se em História a distância EAD com flexibilidade e qualidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Crítica de fontes em arquivo histórico</t>
+  </si>
+  <si>
+    <t>Historiador de cerca de 30 anos, homem de pele clara, cabelo ondulado, camisa e colete, luvas de algodão, atenção ao documento.</t>
+  </si>
+  <si>
+    <t>Sala de arquivo contemporânea brasileira, mesa, caixas de acervo, janela com persiana, espaço sóbrio, sem quadro escolar.</t>
+  </si>
+  <si>
+    <t>documento antigo fechado, lupa, luvas, caderno, caixa de acervo</t>
+  </si>
+  <si>
+    <t>Examina o documento fechado com a lupa e anota no caderno, sentado à direita.</t>
+  </si>
+  <si>
+    <t>Formato quadrado 1:1, enquadramento médio, personagem sentado à direita, região inferior esquerda livre, nenhum rosto, mão ou objeto importante na região inferior esquerda, iluminação publicitária natural suave, separação clara entre assunto e fundo.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; giz; linha do tempo legível; toga; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Historiador, homem de pele clara, cerca de 30 anos, colete e luvas, examinando o documento fechado com a lupa. Objetos: documento fechado, lupa, luvas, caderno e caixa de acervo. Sem giz, sem linha do tempo, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>gestao-de-turismo-ead-tecnologo</t>
   </si>
   <si>
@@ -7164,6 +7440,9 @@
   </si>
   <si>
     <t>gestao-de-turismo</t>
+  </si>
+  <si>
+    <t>Organize produtos de hospitalidade e lazer, com agenciamento, roteiros e avaliação de potencial turístico.</t>
   </si>
   <si>
     <t>O curso de Gestão de Turismo EAD oferece a titulação de tecnólogo e prepara os alunos para planejar e organizar produtos e serviços relacionados a hospitalidade e lazer, como geri-los e avaliá-los. Além disso, o curso capacita para o desenvolvimento e planejamento de atividades turísticas, agenciamento de viagens, coordenação de transportadoras turísticas, consultoria, podendo também identificar possíveis potenciais turísticos para desenvolvimento local e regional. O curso tem 4 semestres (2 anos) de duração e conta com o conceito 5 de classificação do MEC, juntamente com um material didático digital, com ambiente digital moderno e professores especializados.</t>
@@ -7198,6 +7477,27 @@
     <t>Aprenda a gerir negócios no setor do turismo a distância EAD com qualidade e flexibilidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Montagem de roteiro e agenciamento de viagem</t>
+  </si>
+  <si>
+    <t>Gestora de turismo de cerca de 28 anos, mulher de pele morena, cabelo ondulado solto, camisa e lenço, atenção ao mural de roteiro.</t>
+  </si>
+  <si>
+    <t>Agência de turismo contemporânea brasileira, mural, mesa, janela, fotos de paisagens sem legendas, espaço acessível, sem salão de eventos e sem mapa-múndi diplomático.</t>
+  </si>
+  <si>
+    <t>mural de roteiro com cartões em branco, pastas de hospedagem, caneta, calculadora, fotos sem legendas</t>
+  </si>
+  <si>
+    <t>Fixa um cartão no mural do roteiro e confere a pasta de hospedagem, em pé à direita.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; palco de evento; fita no chão de salão; fileira de bandeiras; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Gestora de turismo, mulher de pele morena, cerca de 28 anos, camisa e lenço, fixando cartão em branco no mural de roteiro. Objetos: mural, pastas, caneta, calculadora e fotos sem legendas. Sem palco, sem bandeiras, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>historia-licenciatura-semipresencial-licenciatura</t>
   </si>
   <si>
@@ -7205,6 +7505,9 @@
   </si>
   <si>
     <t>historia-licenciatura</t>
+  </si>
+  <si>
+    <t>Apresente períodos históricos no ensino básico, com fontes, análise crítica e metodologias educativas.</t>
   </si>
   <si>
     <t>O curso de Licenciatura em História semipresencial da Universidade Cruzeiro do Sul Virtual, com duração de 8 semestres (4 anos), prepara os futuros professores para o ensino de História no ensino fundamental e médio. Os estudantes exploram diversos períodos históricos, desenvolvendo competências em pesquisa histórica, análise crítica de fontes e metodologias educacionais inovadoras. O curso oferece flexibilidade para que os alunos estudem no seu próprio ritmo, utilizando recursos digitais avançados. Ao concluir, os alunos recebem o título de Licenciatura, capacitados para lecionar e contribuir para a formação de uma consciência histórica crítica na sociedade.</t>
@@ -7241,6 +7544,27 @@
     <t>Prepare-se para lecionar História a distância EAD com qualidade e reconhecimento. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Aula com linha do tempo ilustrada e fonte em fac-símile</t>
+  </si>
+  <si>
+    <t>Professora de história de cerca de 24 anos, mulher de pele negra, cabelo box braids, blusa verde, apontando a linha do tempo.</t>
+  </si>
+  <si>
+    <t>Sala de história com mural ilustrado contemporânea brasileira, carteiras, linha do tempo na parede, janelas, sem arquivo de acervo.</t>
+  </si>
+  <si>
+    <t>linha do tempo ilustrada sem escritos, fac-símile fechado, giz, apagador, livros fechados</t>
+  </si>
+  <si>
+    <t>Aponta um recorte da linha do tempo e mostra o fac-símile fechado à turma, em pé à direita.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; luvas de arquivo; caixa de acervo; lupa de pesquisa; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento aberto, personagem na região superior direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Professora de história, mulher de pele negra, cerca de 24 anos, blusa verde, apontando a linha do tempo ilustrada sem escritos. Objetos: linha do tempo, fac-símile fechado, giz, apagador e livros. Sem luvas de arquivo, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>letras-portugues-e-ingles-semipresencial-licenciatura</t>
   </si>
   <si>
@@ -7248,6 +7572,9 @@
   </si>
   <si>
     <t>letras-portugues-e-ingles</t>
+  </si>
+  <si>
+    <t>Desenvolva práticas orais e literárias de inglês na educação básica, com didática e leitura compartilhada.</t>
   </si>
   <si>
     <t>O curso de Letras - Português e Inglês semipresencial da Cruzeiro do Sul Virtual tem como objetivo desenvolver habilidades para que os alunos possam interagir em diversos contextos sociocomunicativos, preparando-se para uma atuação dinâmica e eficaz como professores.Como uma licenciatura, o curso inclui disciplinas como didática, metodologia e práticas de ensino de línguas, assim como o estudo das respectivas literaturas, para uma formação completa e voltada para a prática em sala de aula. Além disso, contempla o estudo aprofundado dos aspectos histórico-culturais da língua inglesa oral e escrita, abrangendo obras de autores clássicos e contemporâneos das literaturas Inglesa, Norte-americana, literatura Africana em Língua Portuguesa e literatura Infantojuvenil.Todo esse conjunto de conhecimentos contribui para a excelência na produção de material didático e na orientação teórico-metodológica oferecida nos cursos de Letras da Cruzeiro do Sul Virtual. Com duração de 8 semestres (4 anos), o curso confere o título de licenciatura.</t>
@@ -7282,6 +7609,27 @@
     <t>Desenvolva habilidades em Português e Inglês a distância EAD com flexibilidade e baixo custo. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Leitura compartilhada e prática oral em sala</t>
+  </si>
+  <si>
+    <t>Professora de inglês de cerca de 27 anos, mulher de pele morena, cabelo cacheado médio, camisa xadrez, livro fechado na mão.</t>
+  </si>
+  <si>
+    <t>Sala de leitura escolar brasileira contemporânea, tapete, almofadas, estante baixa, janela, espaço claro, sem cabines de áudio.</t>
+  </si>
+  <si>
+    <t>livros fechados, fantoche, cartaz ilustrado sem escritos, almofadas, caderno</t>
+  </si>
+  <si>
+    <t>Senta no tapete com o fantoche e mostra o livro fechado ao grupo, à direita da estante.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; bandeiras; inglês legível; pincel e tinteiro; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento aberto, personagem na região superior direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Professora de inglês, mulher de pele morena, cerca de 27 anos, camisa xadrez, no tapete com fantoche e livro fechado. Objetos: livros, fantoche, cartaz ilustrado, almofadas e caderno. Sem bandeiras, sem escritos em inglês, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>podologia-semipresencial-tecnologo</t>
   </si>
   <si>
@@ -7289,6 +7637,9 @@
   </si>
   <si>
     <t>podologia</t>
+  </si>
+  <si>
+    <t>Cuide da prevenção e dos cuidados dos pés, com anatomia, fisiologia e práticas especializadas de bem-estar.</t>
   </si>
   <si>
     <t>O curso de Podologia semipresencial da Cruzeiro do Sul Virtual promove uma formação completa e especializada. Ao longo da graduação, os alunos contam com diversas disciplinas que abrangem bases anatômicas e fisiológicas dos pés, aprendendo a identificar, prevenir e tratar patologias, além de oferecer cuidados estéticos e terapêuticos. Com duração de 4 semestres (2 anos), o currículo inclui anatomia, fisiologia, patologia, microbiologia e farmacologia. Com acesso a laboratórios virtuais e práticas supervisionadas, os estudantes desenvolvem habilidades práticas essenciais.</t>
@@ -7323,6 +7674,27 @@
     <t>Estude Podologia a distância EAD com a mesma qualidade do presencial. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Preparação de kit e observação do modelo anatômico do pé</t>
+  </si>
+  <si>
+    <t>Podóloga de cerca de 32 anos, mulher de pele negra, cabelo preso em coque, jaleco e touca, atenção ao modelo.</t>
+  </si>
+  <si>
+    <t>Consultório de podologia contemporâneo brasileiro, cadeira vazia, bancada organizada, iluminação clara, sem spa de luxo.</t>
+  </si>
+  <si>
+    <t>modelo anatômico de pé, kit esterilizado fechado, luvas, gazes, lixeira de procedimentos</t>
+  </si>
+  <si>
+    <t>Alinha o kit fechado e aponta uma estrutura no modelo do pé, em pé à direita da bancada, sem intervir em pessoa.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; diagnóstico; cura; tratamento; spa; pé ferido; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Podóloga, mulher de pele negra, cerca de 32 anos, jaleco e touca, apontando o modelo anatômico do pé ao lado do kit fechado. Objetos: modelo de pé, kit fechado, luvas, gazes e lixeira. Sem spa, sem ferimento, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>computacao-na-nuvem-ead-tecnologo</t>
   </si>
   <si>
@@ -7330,6 +7702,9 @@
   </si>
   <si>
     <t>computacao-na-nuvem</t>
+  </si>
+  <si>
+    <t>Implemente infraestrutura e aplicações em nuvem, com conectividade, dados e modelos de gestão de TI.</t>
   </si>
   <si>
     <t>O curso de Computação em Nuvem EAD busca capacitar os estudantes para dominar técnicas e ferramentas no segmento da Tecnologia da Informação, fornecendo diversos conhecimentos da área, incluindo fundamentos teóricos da computação em nuvem e aplicação prática das mais avançadas soluções tecnológicas. Com disciplinas como Conectividade e Dados da Nuvem; IoT e Stream de Dados; Modelos de Gestão de TI e Técnicas de Desenvolvimento de Algoritmos, o curso confere a titulação de tecnólogo em Computação em Nuvem e tem duração de 4 semestres (2 anos).</t>
@@ -7367,6 +7742,27 @@
     <t>Desenvolva habilidades em Computação na Nuvem a distância EAD com qualidade e reconhecimento. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Desenho de arquitetura de nuvem em camadas</t>
+  </si>
+  <si>
+    <t>Arquiteto de nuvem de cerca de 28 anos, homem de pele clara, cabelo curto, camisa social, atenção ao diagrama na mesa.</t>
+  </si>
+  <si>
+    <t>Sala de operações de TI contemporânea brasileira, mesa com diagrama impresso, um monitor apagado, persiana, sem quadro branco de camadas e sem sensores físicos.</t>
+  </si>
+  <si>
+    <t>diagrama de nuvens em branco, adesivos em branco, caneta, notebook fechado, copo</t>
+  </si>
+  <si>
+    <t>Organiza adesivos sobre o diagrama impresso de nuvens, sentado à direita da mesa.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; holograma; protoboard; sensores; capuz; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Arquiteto de nuvem, homem de pele clara, cerca de 28 anos, camisa social, organizando adesivos sobre o diagrama impresso de nuvens. Objetos: diagrama, adesivos, caneta, notebook fechado e copo. Sem sensores, sem holograma, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>ciencia-de-dados-ead-tecnologo</t>
   </si>
   <si>
@@ -7374,6 +7770,9 @@
   </si>
   <si>
     <t>ciencia-de-dados</t>
+  </si>
+  <si>
+    <t>Modele estatística, algoritmos e programação para extrair conhecimentos que apoiem decisões nas organizações.</t>
   </si>
   <si>
     <t>O curso de Ciências de Dados EAD forma profissionais inovadores em diversos contextos, fornecendo embasamento teórico e prático em áreas como negócios, estatística, algoritmos, programação, banco de dados e inteligência artificial. O curso qualifica o aluno para construir sistemas, escolher componentes, direcionar estratégias, fazer migrações e desenvolver ambientes seguros.Com duração de 4 semestres (2 anos), o curso confere a titulação de tecnólogo em Ciências de Dados.Assim, ao se formar, o cientista de dados estará apto a trabalhar ferramentas matemáticas, estatísticas e computacionais voltadas a auxiliar no processo de extração de conhecimentos a partir de dados, que auxiliam nas tomadas de decisões das organizações.</t>
@@ -7408,6 +7807,27 @@
     <t>Aprenda Ciência de Dados com qualidade e flexibilidade. Vestibular On-line em EAD líder. Bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Modelagem estatística e escolha de componentes</t>
+  </si>
+  <si>
+    <t>Cientista de dados de cerca de 29 anos, mulher de pele morena, cabelo liso longo, camisa azul e cardigan, atenção ao caderno de fórmulas.</t>
+  </si>
+  <si>
+    <t>Sala de modelagem em empresa brasileira contemporânea, lousa com símbolos matemáticos ilegíveis, um monitor com dispersão abstrata, persiana, sem mural de calor e sem cilindros de banco.</t>
+  </si>
+  <si>
+    <t>lousa com símbolos, caderno de fórmulas, calculadora científica, caneta, monitor com dispersão</t>
+  </si>
+  <si>
+    <t>Copia um símbolo da lousa para o caderno e confere a dispersão no monitor, sentada à direita.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; três monitores de calor; cilindros de backup; holograma; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Cientista de dados, mulher de pele morena, cerca de 29 anos, cardigan, copiando símbolos da lousa para o caderno e olhando a dispersão no monitor. Objetos: lousa, caderno, calculadora científica, caneta e monitor. Sem mural de calor, sem cilindros, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>administracao-publica-ead-bacharelado</t>
   </si>
   <si>
@@ -7415,6 +7835,9 @@
   </si>
   <si>
     <t>administracao-publica</t>
+  </si>
+  <si>
+    <t>Formule políticas e projetos de interesse público, com análise quantitativa e fundamentos do Estado.</t>
   </si>
   <si>
     <t>O curso de Administração Pública EAD da Cruzeiro do Sul Virtual prepara os alunos para enfrentar desafios do setor público. Durante a graduação, eles aprendem a identificar e resolver problemas de interesse público, o que os tornará aptos a formular e implementar políticas e projetos, utilizando métodos quantitativos para análise de dados. A formação abrange disciplinas como administração, contabilidade, política, economia, direito, filosofia, sociologia, e tecnologia da informação e comunicação.Os graduados saem com uma compreensão completa das estratégias e métodos de gestão pública, prontos para atuar com uma visão ampla dos fundamentos do Estado. Com duração de 8 semestres (4 anos), o curso oferece o título de bacharel em Administração Pública.</t>
@@ -7455,6 +7878,27 @@
     <t>Desenvolva sua carreira na Administração Pública a baixo custo. Vestibular Online em EAD reconhecida. Bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Planejamento estratégico e orçamento institucional</t>
+  </si>
+  <si>
+    <t>Administradora pública de cerca de 32 anos, mulher de pele negra, cabelo crespo curto, blazer grafite, atenção ao painel de metas vazio.</t>
+  </si>
+  <si>
+    <t>Sala de planejamento em órgão público brasileiro contemporâneo, mesa oval, painel, persiana, espaço institucional sóbrio, sem fila de atendimento e sem tribuna.</t>
+  </si>
+  <si>
+    <t>pastas orçamentárias, gráfico de colunas sem legendas, caneta, copos, notebook fechado</t>
+  </si>
+  <si>
+    <t>Compara tabelas impressas sem números legíveis e anota no caderno orçamentário, sentada à direita.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; fita de fila; totens; palanque; bandeiras; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Administradora pública, mulher de pele negra, cerca de 32 anos, blazer grafite, comparando tabelas impressas e anotando no caderno. Objetos: pastas, gráfico sem legendas, caneta, copos e notebook fechado. Sem fila, sem totens, sem palanque, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>negocios-imobiliarios-ead-tecnologo</t>
   </si>
   <si>
@@ -7462,6 +7906,9 @@
   </si>
   <si>
     <t>negocios-imobiliarios</t>
+  </si>
+  <si>
+    <t>Avalie imóveis e administre condomínios com técnicas de gestão, direito imobiliário e negociação estratégica.</t>
   </si>
   <si>
     <t>O curso de Negócios Imobiliários EAD da Cruzeiro do Sul Virtual é reconhecido pelo Conselho Federal dos Corretores de Imóveis (COFECI) e forma profissionais qualificados para avaliar imóveis, negociações de compra e administração de condomínio. O profissional será apto a aplicar técnicas de gestão, direito imobiliário, corretagem e avaliação imobiliária, traçando estratégias de administração e negociação. Com duração de 4 semestres (2 anos), o curso confere o título de tecnólogo em Negócios Imobiliários.</t>
@@ -7496,6 +7943,27 @@
     <t>Aprenda sobre Negócios Imobiliários a distância EAD com flexibilidade e qualidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Avaliação comparativa de plantas de apartamento</t>
+  </si>
+  <si>
+    <t>Analista imobiliário de cerca de 31 anos, homem de pele morena, cabelo curto, camisa social sem gravata, atenção às plantas.</t>
+  </si>
+  <si>
+    <t>Escritório funcional em prédio residencial brasileiro, mesa, janela para fachada comum, espaço acessível, sem cobertura de luxo e sem entrega de chaves.</t>
+  </si>
+  <si>
+    <t>plantas baixas sem nomes, trena, pasta de avaliação, calculadora, caneta</t>
+  </si>
+  <si>
+    <t>Compara duas plantas baixas e confere a trena sobre a mesa, sentado à direita.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; mansão; chave na mão do cliente; aperto de mãos; capacete de obra; ambiente de luxo ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Analista imobiliário, homem de pele morena, cerca de 31 anos, camisa social, comparando duas plantas baixas e conferindo a trena. Objetos: plantas, trena, pasta, calculadora e caneta. Sem mansão, sem chaves, sem aperto de mãos, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>seguranca-do-trabalho-ead-tecnologo</t>
   </si>
   <si>
@@ -7503,6 +7971,9 @@
   </si>
   <si>
     <t>seguranca-do-trabalho</t>
+  </si>
+  <si>
+    <t>Identifique riscos ocupacionais e organize medidas preventivas para a saúde e a segurança no trabalho.</t>
   </si>
   <si>
     <t>O curso de Segurança no Trabalho EAD da Cruzeiro do Sul Virtual forma profissionais capazes para atuar na prevenção de acidentes e doenças ocupacionais nas diversas áreas de trabalho, desenvolvendo habilidades e competências para identificar riscos ambientais, criação de planos preventivos e implementação de medidas que garantam a saúde e segurança dos trabalhadores. Com disciplinas como Saúde do trabalhador, Doenças ocupacionais, Gestão de pessoas, Psicologia do trabalho e Auditoria, laudos e perícias, o curso tem duração de 6 semestres (3 anos), titulação de tecnologia e conceito 4 na classificação do MEC.</t>
@@ -7536,6 +8007,27 @@
     <t>Desenvolva habilidades em Segurança do Trabalho a distância EAD com flexibilidade e qualidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Inspeção preventiva de EPIs e sinalização de risco</t>
+  </si>
+  <si>
+    <t>Técnica de segurança de cerca de 30 anos, mulher de pele clara, cabelo preso, colete e capacete, prancheta na mão.</t>
+  </si>
+  <si>
+    <t>Passarela de indústria brasileira contemporânea, EPIs alinhados, piso sinalizado, iluminação industrial, espaço organizado, sem acidente e sem arma.</t>
+  </si>
+  <si>
+    <t>prancheta de inspeção em branco, capacete extra, luvas, protetor auricular, fita zebrada enrolada</t>
+  </si>
+  <si>
+    <t>Confere o capacete extra e registra a inspeção na prancheta, em pé à direita da passarela.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; acidente; trabalhador ferido; sangue; arma; viatura; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio-aberto, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Técnica de segurança, mulher de pele clara, cerca de 30 anos, colete e capacete, conferindo EPI e anotando na prancheta. Objetos: prancheta em branco, capacete extra, luvas, protetor auricular e fita enrolada. Sem acidente, sem ferimento, sem arma, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>administracao-ead-bacharelado</t>
   </si>
   <si>
@@ -7543,6 +8035,9 @@
   </si>
   <si>
     <t>administracao</t>
+  </si>
+  <si>
+    <t>Dirija a gestão estratégica de negócios, com pessoas, finanças, logística e competitividade organizacional.</t>
   </si>
   <si>
     <t>O curso de Bacharelado em Administração EAD da Cruzeiro do Sul Virtual é a escolha ideal para quem busca uma formação de excelência com a flexibilidade do ensino a distância. Com duração de 8 semestres (4 anos), a graduação prepara você para os desafios do mercado corporativo moderno.</t>
@@ -7578,6 +8073,27 @@
     <t>Estude Administração a distância com flexibilidade e qualidade. Vestibular Online em uma instituição de referência. Bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Reunião de gestão estratégica entre áreas</t>
+  </si>
+  <si>
+    <t>Administrador de cerca de 34 anos, homem de pele negra, cabelo curto, camisa e blazer simples, apontando o painel de áreas.</t>
+  </si>
+  <si>
+    <t>Sala de diretoria acessível em empresa brasileira contemporânea, mesa longa, painel com quatro quadrantes vazios, janela, sem papel pardo de fluxograma.</t>
+  </si>
+  <si>
+    <t>painel de quadrantes em branco, pastas de áreas, caneta, jarra, notebook fechado</t>
+  </si>
+  <si>
+    <t>Aponta um quadrante vazio e distribui pastas de áreas, em pé à direita da mesa.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; papel pardo de gargalos; foguete; aperto de mãos; fila de atendimento; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Administrador, homem de pele negra, cerca de 34 anos, blazer simples, apontando quadrante vazio e distribuindo pastas. Objetos: painel, pastas, caneta, jarra e notebook fechado. Sem fluxograma, sem foguete, sem aperto de mãos, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>ciencias-biologicas-licenciatura-semipresencial-licenciatura</t>
   </si>
   <si>
@@ -7585,6 +8101,9 @@
   </si>
   <si>
     <t>ciencias-biologicas-licenciatura</t>
+  </si>
+  <si>
+    <t>Ensine evolução e conservação em estufa escolar, com amostras vegetais e práticas de educação ambiental.</t>
   </si>
   <si>
     <t>O curso de Licenciatura em Ciências Biológicas semipresencial, estudará a vida existente no planeta, através de um olhar científico, contando com laboratórios modernos e equipados, com aulas e visitas técnicas. Sob a visão da educação, o licenciado em Ciências Biológicas pela universidade Cruzeiro do Sul Virtual será estimulado a realizar projetos e pesquisas sobre meio ambiente, saúde e biotecnologia, com foco na conservação e preservação da biodiversidade. Com duração de 8 semestres (4 anos), o profissional será capaz de compreender a complexidade sobre as vidas existentes no planeta, processos evolutivos e muito mais. O curso possui conceito 4 no MEC e confere o título de licenciatura em Ciências Biológicas.</t>
@@ -7620,6 +8139,27 @@
     <t>Prepare-se para ensinar Ciências Biológicas com flexibilidade do EAD e qualidade. Bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Aula de biodiversidade com amostras vegetais</t>
+  </si>
+  <si>
+    <t>Professora de biologia de cerca de 24 anos, mulher de pele morena, cabelo cacheado solto, camisa floral e avental, mostrando a planta.</t>
+  </si>
+  <si>
+    <t>Estufa escolar brasileira contemporânea, bancadas com vasos, mangueira, luz de manhã, espaço de aula ao ar coberto, sem trilha de reserva.</t>
+  </si>
+  <si>
+    <t>vaso com planta, lupa, béquer, giz, bandeja de folhas</t>
+  </si>
+  <si>
+    <t>Mostra a folha na lupa para a turma e aponta o vaso, em pé à direita da bancada, quadro apagado.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; rede entomológica de campo; microscópio clínico; animal ferido; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento aberto, personagem na região superior direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Professora de biologia, mulher de pele morena, cerca de 24 anos, camisa floral e avental, mostrando a folha na lupa à turma na estufa escolar. Objetos: vaso, lupa, béquer, giz e bandeja de folhas. Sem rede de campo, sem microscópio clínico, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>engenharia-mecatronica-semipresencial-bacharelado</t>
   </si>
   <si>
@@ -7627,6 +8167,9 @@
   </si>
   <si>
     <t>engenharia-mecatronica</t>
+  </si>
+  <si>
+    <t>Automatize linhas produtivas com robôs, sensores de precisão e controle de células industriais robotizadas.</t>
   </si>
   <si>
     <t>O curso de Engenharia Mecatrônica Semipresencial da Cruzeiro do Sul Virtual forma engenheiros capacitados para liderar a Indústria 4.0. Com foco em inovação e eficiência produtiva, a graduação integra os pilares da Engenharia Mecânica, Eletrônica e Computação, preparando o aluno para desenvolver sistemas de automação industrial e robótica avançada.</t>
@@ -7661,6 +8204,27 @@
     <t>Estude Engenharia Mecatrônica a distância EAD com a mesma qualidade do presencial. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Ajuste de célula robótica de automação</t>
+  </si>
+  <si>
+    <t>Engenheiro mecatrônico de cerca de 27 anos, homem de pele negra, cabelo black curto, macacão cinza, teach pendant na mão.</t>
+  </si>
+  <si>
+    <t>Célula de automação em indústria brasileira contemporânea, braço robótico parado, grade de proteção, piso limpo, sem caixa de engrenagens solta e sem quadro elétrico aberto.</t>
+  </si>
+  <si>
+    <t>braço robótico, teach pendant, chave allen, cone de segurança, prancheta</t>
+  </si>
+  <si>
+    <t>Ajusta a posição do braço robótico e confere o teach pendant, em pé à direita da grade.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; holograma; capuz; engrenagem como único objeto; fiação exposta; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio-aberto, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Engenheiro mecatrônico, homem de pele negra, cerca de 27 anos, macacão, ajustando o braço robótico e conferindo o teach pendant. Objetos: braço robótico, teach pendant, chave allen, cone e prancheta. Sem holograma, sem engrenagens soltas, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>sistemas-para-internet-ead-tecnologo</t>
   </si>
   <si>
@@ -7668,6 +8232,9 @@
   </si>
   <si>
     <t>sistemas-para-internet</t>
+  </si>
+  <si>
+    <t>Construa websites e aplicações online, com programação web, bancos de dados e integração de sistemas.</t>
   </si>
   <si>
     <t>O curso de Sistemas para Internet EAD capacita profissionais para desenvolver soluções tecnológicas voltadas para a web. Com foco no desenvolvimento, instalação de bancos de dados e aplicações online, o currículo engloba disciplinas como programação web, design de interação, banco de dados, segurança de sistemas e gestão da tecnologia da informação. Os alunos adquirem habilidades em desenvolvimento de websites dinâmicos, aplicativos web, e-commerce, marketing digital, e integração de sistemas online. Com duração de 4 semestres (2 anos), conceito 5 na classificação do MEC e conferindo o título de tecnólogo, o curso prepara os graduandos para o mercado de trabalho em grandes empresas.</t>
@@ -7703,6 +8270,27 @@
     <t>Desenvolva habilidades em Sistemas para Internet a distância EAD com flexibilidade e qualidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Montagem de páginas e navegação de aplicação web</t>
+  </si>
+  <si>
+    <t>Desenvolvedora web de cerca de 24 anos, mulher de pele clara, cabelo ondulado castanho, moletom verde, atenção ao navegador.</t>
+  </si>
+  <si>
+    <t>Sala de produto digital em agência pequena brasileira, dois monitores com blocos de layout, persiana, espaço contemporâneo, sem coworking e sem mesa alta doméstica.</t>
+  </si>
+  <si>
+    <t>notebook, mouse, fone, caderno de esboço de tela em branco, copo</t>
+  </si>
+  <si>
+    <t>Arrasta blocos no layout do navegador e confere o esboço de tela em branco, sentada à direita, tela sem escritos.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; código de servidor; holograma; capuz; tapete de corte; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Desenvolvedora web, mulher de pele clara, cerca de 24 anos, moletom verde, arrastando blocos no layout do notebook. Tela com blocos coloridos, sem escritos. Objetos: notebook, mouse, fone, caderno em branco e copo. Sem terminal de servidor, sem mural de jornada, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>fisioterapia-semipresencial-bacharelado</t>
   </si>
   <si>
@@ -7710,6 +8298,9 @@
   </si>
   <si>
     <t>fisioterapia</t>
+  </si>
+  <si>
+    <t>Oriente exercícios de mobilidade e reabilitação funcional, com anatomia, fisiologia e biomecânica do movimento.</t>
   </si>
   <si>
     <t>A graduação de Fisioterapia semipresencial da Cruzeiro do Sul Virtual, fornece aos estudantes um ensino pautado na promoção de saúde e bem-estar dos indivíduos, com base em uma compreensão profunda da anatomia humana. Ao longo do curso, os alunos são convidados a refletir e analisar disciplinas imersivas, como anatomia, fisiologia, biomecânica e cinesiologia, o que consolida fortes fundamentos para o completo entendimento do corpo humano. A Cruzeiro do Sul Virtual promove conhecimentos robustos, com o objetivo de transformar seus alunos em profissionais altamente competentes para diagnosticar, prevenir e corrigir distúrbios motores, além de desenvolver técnicas de reabilitação física e exercer uma função essencial na elevação da qualidade de vida das pessoas.</t>
@@ -7744,6 +8335,27 @@
     <t>Estude Fisioterapia a distância EAD com a mesma qualidade do presencial. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Orientação de mobilidade em barras paralelas</t>
+  </si>
+  <si>
+    <t>Fisioterapeuta de cerca de 30 anos, mulher de pele negra, cabelo em box braids, jaleco esportivo e calça, postura de orientação.</t>
+  </si>
+  <si>
+    <t>Sala de reabilitação contemporânea brasileira, barras paralelas, colchonete, janela, espaço digno, sem cozinha terapêutica e sem espelho de articulação.</t>
+  </si>
+  <si>
+    <t>barras paralelas, bola de exercícios, faixa elástica, cronômetro, colchonete</t>
+  </si>
+  <si>
+    <t>Guia os pés de uma pessoa adulta nas barras e segura a faixa elástica, em pé à direita, sem aplicar diagnóstico.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; diagnóstico; cura; tratamento; utensílio de cozinha; espelho de fala; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Fisioterapeuta, mulher de pele negra, cerca de 30 anos, jaleco esportivo, guiando a pessoa nas barras paralelas. Objetos: barras, bola, faixa elástica, cronômetro e colchonete. Sem cozinha terapêutica, sem espelho de fala, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>coaching-e-mentoring-ead-tecnologo</t>
   </si>
   <si>
@@ -7751,6 +8363,9 @@
   </si>
   <si>
     <t>coaching-e-mentoring</t>
+  </si>
+  <si>
+    <t>Conduza conversas de desenvolvimento de liderança e desempenho, com acompanhamento de metas e relações de equipe.</t>
   </si>
   <si>
     <t>O curso de Coaching e Mentoring EAD da Cruzeiro do Sul Virtual foi pensado para capacitação do profissional através de conhecimentos sobre o comportamento humano, a fim de auxiliar pessoas de diversas áreas e cargos a atingirem suas metas. O coach graduado pela Cruzeiro do Sul Virtual desempenha a implementação de mudanças organizacionais e seus funcionários, fazendo o uso de ferramentas para que o senso de liderança, autonomia e bem-estar organizacional seja expandido, gerenciando o desempenho e a melhora das relações interpessoais. Com duração de 4 semestres (2 anos), o curso confere o título de tecnólogo em Coaching e Mentoring.</t>
@@ -7785,6 +8400,27 @@
     <t>Aprimore suas habilidades em Coaching e Mentoring a distância EAD com qualidade e reconhecimento. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Sessão de acompanhamento de metas e liderança</t>
+  </si>
+  <si>
+    <t>Coach de cerca de 33 anos, homem de pele clara, cabelo curto, óculos e pulôver, caderno de perguntas na mão.</t>
+  </si>
+  <si>
+    <t>Pátio interno de empresa brasileira contemporânea, bancos, planta, luz da manhã, conversa em pé ao ar livre, sem sala de entrevistas.</t>
+  </si>
+  <si>
+    <t>caderno de perguntas, cartões de meta em branco, caneta, copo, pasta</t>
+  </si>
+  <si>
+    <t>Caminha ao lado da pessoa e mostra um cartão de meta em branco, em pé à direita do corredor.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; aperto de mãos; foguete; cifrão; palco; divã; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Coach, homem de pele clara, cerca de 33 anos, pulôver e óculos, no pátio mostrando cartão de meta em branco. Objetos: caderno, cartões em branco, caneta, copo e pasta. Sem aperto de mãos, sem foguete, sem palco, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>internet-das-coisas-ead-tecnologo</t>
   </si>
   <si>
@@ -7792,6 +8428,9 @@
   </si>
   <si>
     <t>internet-das-coisas</t>
+  </si>
+  <si>
+    <t>Conecte sensores e dispositivos a sistemas organizacionais, com testes de automação e coleta de dados.</t>
   </si>
   <si>
     <t>O Tecnólogo em Internet das Coisas no formato EAD da Cruzeiro do Sul Virtual garante fornecer aos estudantes competências para atividades técnicas e científicas, os tornando aptos a projetar, analisar, desenvolver e testar sistemas para internet das coisas, utilizando tecnologias e conceitos modernos, e dessa forma, aprimorando a eficiência dos sistemas organizacionais. Além do mais, o curso da Cruzeiro do Sul Virtual tem duração de 4 semestres (2 anos) e conta com matriz curricular moderna e alinhada com o mercado, assim como atividades formativas e práticas.</t>
@@ -7825,6 +8464,27 @@
     <t>Estude sobre a Internet das Coisas a distância EAD com a mesma qualidade do presencial. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Teste de sensores conectados em bancada</t>
+  </si>
+  <si>
+    <t>Desenvolvedora de IoT de cerca de 25 anos, mulher de pele morena, cabelo cacheado curto, camisa e avental de bancada, atenção ao sensor.</t>
+  </si>
+  <si>
+    <t>Bancada de protótipos IoT em laboratório brasileiro contemporâneo, cabos organizados, janela, espaço técnico, sem desenho de nuvem no quadro.</t>
+  </si>
+  <si>
+    <t>placa com sensores, cabo, display numérico genérico, protoboard, chave de fenda</t>
+  </si>
+  <si>
+    <t>Conecta o cabo ao sensor e observa o display numérico, sentada à direita da bancada.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; holograma; nuvens desenhadas no quadro; capuz; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Desenvolvedora de IoT, mulher de pele morena, cerca de 25 anos, avental de bancada, conectando o cabo ao sensor. Objetos: placa com sensores, cabo, display, protoboard e chave. Sem desenho de nuvem, sem holograma, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>empreendedorismo-ead-tecnologo</t>
   </si>
   <si>
@@ -7832,6 +8492,9 @@
   </si>
   <si>
     <t>empreendedorismo</t>
+  </si>
+  <si>
+    <t>Modele planos de um empreendimento acessível, com gestão, finanças, marketing, inovação e liderança.</t>
   </si>
   <si>
     <t>O curso de Empreendedorismo EAD da Cruzeiro do Sul Virtual, com duração de 4 semestres, confere o título de Tecnólogo e possui conceito 4 na classificação do MEC. Este curso prepara os estudantes para identificar oportunidades de negócio, desenvolver planos estratégicos e gerenciar empresas de forma inovadora e sustentável. Através de uma abordagem prática e teórica, os alunos adquirem competências essenciais em gestão, marketing, finanças e liderança, capacitando-se para atuar em diversos setores do mercado e lançar seus próprios empreendimentos.</t>
@@ -7867,6 +8530,27 @@
     <t>Desenvolva habilidades em Empreendedorismo EAD com flexibilidade e qualidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Canvas de negócio e planejamento financeiro simples</t>
+  </si>
+  <si>
+    <t>Empreendedor de cerca de 29 anos, homem de pele negra, cabelo crespo curto, camisa jeans, atenção ao canvas.</t>
+  </si>
+  <si>
+    <t>Pequena oficina de ateliê brasileiro contemporâneo, mesa, prateleira de produtos genéricos, janela, espaço acessível, sem escritório de luxo.</t>
+  </si>
+  <si>
+    <t>canvas com blocos vazios, calculadora, caderno, caneta, amostras genéricas</t>
+  </si>
+  <si>
+    <t>Preenche um bloco vazio do canvas e confere a calculadora, sentada à direita da mesa.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; foguete; aperto de mãos; cifrão; startup de luxo; ambiente precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Empreendedor, homem de pele negra, cerca de 29 anos, camisa jeans, preenchendo bloco vazio do canvas em ateliê simples. Objetos: canvas, calculadora, caderno, caneta e amostras. Sem foguete, sem aperto de mãos, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>engenharia-civil-semipresencial-bacharelado</t>
   </si>
   <si>
@@ -7874,6 +8558,9 @@
   </si>
   <si>
     <t>engenharia-civil</t>
+  </si>
+  <si>
+    <t>Planeje estruturas, fundações e serviços de obras, com vistoria de edificações e sistemas de infraestrutura.</t>
   </si>
   <si>
     <t>O curso de Engenharia Civil semipresencial da Cruzeiro do Sul, fornece uma formação combinada entre teoria e prática, com projetos com foco em uma formação detalhada e completa, alinhados às exigências do mercado da área. Com 10 semestres de duração (5 anos), os alunos são preparados para realizar atividades de planejamento, projeto, direção, vistoria e avaliação de obras e serviços relacionados a edificações, sistemas de transporte, abastecimento de água, drenagem e outros aspectos. O curso oferece a titulação de bacharel em Engenharia Civil.</t>
@@ -7911,6 +8598,27 @@
     <t>Estude Engenharia Civil a distância EAD com a mesma qualidade do presencial. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Vistoria de forma e armadura em canteiro</t>
+  </si>
+  <si>
+    <t>Engenheiro civil de cerca de 30 anos, homem de pele clara, barba curta, óculos de proteção, capacete e colete, prancheta na mão.</t>
+  </si>
+  <si>
+    <t>Canteiro organizado de edifício brasileiro contemporâneo, forma de concreto, armadura visível, piso delimitado, céu claro, sem maquete de ateliê e sem planta de venda.</t>
+  </si>
+  <si>
+    <t>prancheta, trena, capacete, nível de pedreiro, rádio</t>
+  </si>
+  <si>
+    <t>Mede a forma com a trena e anota na prancheta, em pé à direita da armadura.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; maquete de edifício; chave de imóvel; mansão; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio-aberto, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Engenheiro civil, homem de pele clara, cerca de 30 anos, barba, capacete e colete, medindo a forma com a trena. Objetos: prancheta, trena, capacete, nível e rádio. Sem maquete, sem chaves, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>marketing-digital-ead-tecnologo</t>
   </si>
   <si>
@@ -7918,6 +8626,9 @@
   </si>
   <si>
     <t>marketing-digital</t>
+  </si>
+  <si>
+    <t>Defina campanhas e canais digitais, com conteúdo, mídias sociais, publicidade online e leitura de audiência.</t>
   </si>
   <si>
     <t>O curso de Marketing Digital EAD da Cruzeiro do Sul Virtual oferece uma formação completa e atualizada, com disponibilidade das modalidades que contém aulas gravadas e aulas ao vivo, proporcionando flexibilidade e interatividade aos alunos. Com conceito 3 na classificação do MEC, o curso aborda temas como estratégias de marketing online, marketing de conteúdo, gestão de mídias sociais, e análise de dados. Os estudantes têm acesso a uma plataforma virtual com materiais didáticos interativos, videoaulas e suporte de tutores, preparando-os para enfrentar os desafios do mercado de trabalho digital. Com duração de 4 semestres (2 anos), o curso confere o título de Tecnólogo em Marketing Digital.</t>
@@ -7951,6 +8662,27 @@
     <t>Desenvolva habilidades em Marketing Digital a distância EAD com flexibilidade e qualidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Matriz de canais digitais e leitura de audiência</t>
+  </si>
+  <si>
+    <t>Analista de marketing digital de cerca de 26 anos, mulher de pele clara, cabelo curto ondulado, blazer mostarda, atenção ao mural de canais.</t>
+  </si>
+  <si>
+    <t>Sala de planejamento digital contemporânea brasileira, mural, mesa, janela, espaço acessível, sem tripé de influenciador e sem gôndola.</t>
+  </si>
+  <si>
+    <t>mural de canais com cartões em branco, notebook com gráfico abstrato, caneta, tablet, copo</t>
+  </si>
+  <si>
+    <t>Move um cartão no mural de canais e confere o gráfico no notebook, em pé à direita.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; ring light; tripé; gôndola; mesa de luz de peças; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Analista de marketing digital, mulher de pele clara, cerca de 26 anos, blazer mostarda, movendo cartão em branco no mural de canais. Objetos: mural, notebook com gráfico abstrato, caneta, tablet e copo. Sem tripé, sem ring light, sem gôndola, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>formacao-pedagogica-letras-port-e-ing-semipresencial-licenciatura</t>
   </si>
   <si>
@@ -7958,6 +8690,9 @@
   </si>
   <si>
     <t>formacao-pedagogica-letras-port-e-ing</t>
+  </si>
+  <si>
+    <t>Organize sequências didáticas bilíngues de português e inglês para quem já possui graduação e atua na formação docente.</t>
   </si>
   <si>
     <t xml:space="preserve">O curso de Formação Pedagógica em Letras (Português e Inglês) da Cruzeiro do Sul Virtual está disponível no formato Semipresencial e é destinado especificamente a alunos que já possuem uma graduação prévia em Pedagogia. Ao longo da formação, o curso foca em proporcionar o domínio das línguas portuguesa e inglesa, bem como de suas respectivas literaturas, despertando um questionamento crítico e reflexivo acerca da linguagem e da cultura.
@@ -7990,6 +8725,27 @@
     <t>Faça Formação Pedagógica em Letras Português e Inglês semipresencial na Cruzeiro do Sul Virtual e habilite-se para lecionar idiomas no Ensino Fundamental e Médio.</t>
   </si>
   <si>
+    <t>Elaboração de sequência didática bilíngue</t>
+  </si>
+  <si>
+    <t>Formadora pedagógica de cerca de 35 anos, mulher de pele morena, cabelo cacheado preso, camisa e saia, atenção à lousa de planejamento.</t>
+  </si>
+  <si>
+    <t>Sala de formação continuada de docentes brasileira contemporânea, mesa de reunião, lousa com duas colunas vazias, janela, colegas adultos ao fundo, sem turma infantil.</t>
+  </si>
+  <si>
+    <t>lousa de duas colunas, cartões de estratégia em branco, dois livros fechados de cores distintas, pasta de formação, canetão</t>
+  </si>
+  <si>
+    <t>Fixa cartões de estratégia nas duas colunas da lousa e folheia a pasta de formação, em pé à direita.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; laminadora; recorte; artesanato; aula infantil; giz no quadro de turma; bandeiras; inglês legível; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Formadora pedagógica, mulher de pele morena, cerca de 35 anos, camisa e saia, fixando cartões de estratégia em branco nas duas colunas da lousa. Objetos: lousa de duas colunas, cartões em branco, dois livros fechados, pasta de formação e canetão. Sem laminadora, sem recorte, sem turma infantil, sem bandeiras, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>desenvolvimento-back-end-ead-tecnologo</t>
   </si>
   <si>
@@ -7997,6 +8753,9 @@
   </si>
   <si>
     <t>desenvolvimento-back-end</t>
+  </si>
+  <si>
+    <t>Estruture a lógica, a segurança, as regras de negócio e as integrações que sustentam sites e aplicações.</t>
   </si>
   <si>
     <t>O curso de Desenvolvedor de Back-End EAD da Cruzeiro do Sul Virtual capacita profissionais para criar e manter códigos e comandos que fazem dispositivos e serviços web funcionarem. Utilizando linguagens de programação, o desenvolvedor de Back-End constrói a estrutura que suporta as ações das máquinas, garantindo o funcionamento adequado de sites e aplicações. Com uma base teórica sólida em computação, números e raciocínio lógico, esses profissionais são essenciais para a manutenção de sistemas eficientes e seguros. O curso, com duração de 4 semestres (2 anos), oferece a titulação de tecnólogo em Desenvolvimento de Back-End e apresenta um plano pedagógico atualizado, alinhado às exigências do mercado. Utilizando tecnologias avançadas, a formação proporciona aos alunos conhecimentos técnicos específicos de programação e inclui laboratórios virtuais para a aplicação prática da teoria, preparando-os para o mercado de trabalho.</t>
@@ -8030,6 +8789,30 @@
     <t>Desenvolva habilidades em Desenvolvimento Back-End EAD com qualidade e flexibilidade. Vestibular On-line com bolsas de até 100%!</t>
   </si>
   <si>
+    <t>Organização de serviços, regras e integração de dados</t>
+  </si>
+  <si>
+    <t>Desenvolvedor back-end de cerca de 27 anos, homem de pele negra, cabelo crespo curto, camisa preta, atenção aos dois monitores.</t>
+  </si>
+  <si>
+    <t>Sala técnica contemporânea brasileira, dois monitores com blocos de código ilegíveis, persiana, espaço sóbrio, sem layout de página e sem mural de jornada.</t>
+  </si>
+  <si>
+    <t>dois monitores, teclado, caderno de regras, cabo de rede, copo</t>
+  </si>
+  <si>
+    <t>Compara blocos nos dois monitores e anota uma regra no caderno, sentado à direita, telas sem escritos legíveis.</t>
+  </si>
+  <si>
+    <t>Formato quadrado 1:1, enquadramento médio, personagem sentado à direita, região inferior esquerda livre, nenhum rosto, mão ou objeto importante na região inferior esquerda, iluminação publicitária suave, separação clara entre assunto e fundo.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; layout de site colorido; holograma; capuz; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Desenvolvedor back-end, homem de pele negra, cerca de 27 anos, camisa preta, comparando dois monitores com blocos ilegíveis. Objetos: dois monitores, teclado, caderno, cabo e copo. Sem layout de página, sem mural de jornada, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
+  </si>
+  <si>
     <t>sistemas-de-informacao-ead-bacharelado</t>
   </si>
   <si>
@@ -8037,6 +8820,9 @@
   </si>
   <si>
     <t>sistemas-de-informacao</t>
+  </si>
+  <si>
+    <t>Coordene a integração de sistemas e informações entre áreas, com arquitetura empresarial, projetos e segurança da informação.</t>
   </si>
   <si>
     <t>O Bacharelado de Sistemas da Informação EAD da Cruzeiro do Sul Virtual, tem como principal objetivo fornecer uma formação de alta qualidade para seus alunos. O curso proporciona conhecimentos avançados para que os estudantes aprendam a projetar, estruturar, implementar e coordenar sistemas computacionais. Com uma perspectiva integrada entre TI e inovação de soluções, o curso engloba conteúdos essenciais, como redes de computadores, inteligência artificial, programação, banco de dados e gestão de projetos. Com o vasto conhecimento adquirido ao longo do curso, principalmente nas áreas de análise e resolução de problemas tecnológicos, organização de dados e segurança cibernética, os graduados estarão à frente no mercado e atualizados com a inovação das tecnologias no Brasil e no mundo.</t>
@@ -8070,6 +8856,27 @@
   </si>
   <si>
     <t>Prepare-se para atuar em Sistemas de Informação a distância EAD com qualidade e reconhecimento. Vestibular On-line com bolsas de até 100%!</t>
+  </si>
+  <si>
+    <t>Integração de sistemas empresariais entre áreas</t>
+  </si>
+  <si>
+    <t>Analista de sistemas de informação de cerca de 32 anos, mulher de pele clara, cabelo castanho em ondas, camisa social e blazer, atenção aos blocos na mesa.</t>
+  </si>
+  <si>
+    <t>Sala de integração empresarial contemporânea brasileira, mesa com maquete de blocos, notebook, persiana, espaço de projeto, sem quadro de camadas e sem rack.</t>
+  </si>
+  <si>
+    <t>diagrama físico de blocos coloridos, notebook aberto, pasta de documentação, caneta, fios de ligação</t>
+  </si>
+  <si>
+    <t>Liga dois blocos do diagrama com um fio e confere a documentação no notebook, em pé à direita, telas e folhas sem escritos.</t>
+  </si>
+  <si>
+    <t>Palavras, textos, logotipos, marcas ou marca-d'água; mãos incorretas ou objetos deformados; interfaces flutuantes; cilindros de banco; backup; servidor como cena principal; papel pardo de gargalos; código na tela; holograma; capuz; ambiente luxuoso ou precário.</t>
+  </si>
+  <si>
+    <t>Fotografia publicitária realista em cenário brasileiro contemporâneo, iluminação natural profissional. Composição quadrada 1:1, enquadramento médio, assunto principal à direita, região inferior esquerda livre, sem rostos, mãos ou objetos importantes nessa área, separação clara entre pessoa e fundo. Analista de sistemas de informação, mulher de pele clara, cerca de 32 anos, blazer, ligando dois blocos coloridos do diagrama com um fio e conferindo o notebook. Objetos: diagrama de blocos, notebook, pasta de documentação, caneta e fios. Sem cilindros, sem backup, sem rack, sem palavras visíveis, sem legendas, sem identificações comerciais, sem elementos gráficos sobrepostos, sem marca-d'água, sem mãos anatomicamente incorretas e sem objetos deformados.</t>
   </si>
 </sst>
 </file>
@@ -17350,23 +18157,26 @@
       <c r="G97" t="s">
         <v>158</v>
       </c>
+      <c r="H97" t="s">
+        <v>2015</v>
+      </c>
       <c r="I97" t="s">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="J97" t="s">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="K97" t="s">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="L97" t="s">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="M97" t="s">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="N97" t="s">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="P97" t="s">
         <v>166</v>
@@ -17381,27 +18191,54 @@
         <v>167</v>
       </c>
       <c r="T97" t="s">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="U97" t="s">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="V97" t="s">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="W97" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X97" t="s">
+        <v>2025</v>
+      </c>
+      <c r="Y97" t="s">
+        <v>2026</v>
+      </c>
+      <c r="Z97" t="s">
+        <v>2027</v>
+      </c>
+      <c r="AA97" t="s">
+        <v>2028</v>
+      </c>
+      <c r="AB97" t="s">
+        <v>2029</v>
+      </c>
+      <c r="AC97" t="s">
+        <v>151</v>
+      </c>
+      <c r="AD97" t="s">
+        <v>2030</v>
+      </c>
+      <c r="AE97" t="s">
+        <v>2031</v>
+      </c>
+      <c r="AF97" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="98" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>2024</v>
+        <v>2032</v>
       </c>
       <c r="B98" t="s">
-        <v>2025</v>
+        <v>2033</v>
       </c>
       <c r="C98" t="s">
-        <v>2026</v>
+        <v>2034</v>
       </c>
       <c r="D98" t="s">
         <v>157</v>
@@ -17415,20 +18252,23 @@
       <c r="G98" t="s">
         <v>158</v>
       </c>
+      <c r="H98" t="s">
+        <v>2035</v>
+      </c>
       <c r="I98" t="s">
-        <v>2027</v>
+        <v>2036</v>
       </c>
       <c r="J98" t="s">
-        <v>2028</v>
+        <v>2037</v>
       </c>
       <c r="K98" t="s">
-        <v>2029</v>
+        <v>2038</v>
       </c>
       <c r="M98" t="s">
-        <v>2030</v>
+        <v>2039</v>
       </c>
       <c r="N98" t="s">
-        <v>2031</v>
+        <v>2040</v>
       </c>
       <c r="O98" t="s">
         <v>141</v>
@@ -17446,27 +18286,54 @@
         <v>1534</v>
       </c>
       <c r="T98" t="s">
-        <v>2032</v>
+        <v>2041</v>
       </c>
       <c r="U98" t="s">
-        <v>2033</v>
+        <v>2042</v>
       </c>
       <c r="V98" t="s">
-        <v>2034</v>
+        <v>2043</v>
       </c>
       <c r="W98" s="1" t="s">
         <v>1538</v>
+      </c>
+      <c r="X98" t="s">
+        <v>2044</v>
+      </c>
+      <c r="Y98" t="s">
+        <v>2045</v>
+      </c>
+      <c r="Z98" t="s">
+        <v>2046</v>
+      </c>
+      <c r="AA98" t="s">
+        <v>2047</v>
+      </c>
+      <c r="AB98" t="s">
+        <v>2048</v>
+      </c>
+      <c r="AC98" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD98" t="s">
+        <v>2049</v>
+      </c>
+      <c r="AE98" t="s">
+        <v>2050</v>
+      </c>
+      <c r="AF98" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="99" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>2035</v>
+        <v>2051</v>
       </c>
       <c r="B99" t="s">
-        <v>2036</v>
+        <v>2052</v>
       </c>
       <c r="C99" t="s">
-        <v>2037</v>
+        <v>2053</v>
       </c>
       <c r="D99" t="s">
         <v>35</v>
@@ -17480,23 +18347,26 @@
       <c r="G99" t="s">
         <v>89</v>
       </c>
+      <c r="H99" t="s">
+        <v>2054</v>
+      </c>
       <c r="I99" t="s">
-        <v>2038</v>
+        <v>2055</v>
       </c>
       <c r="J99" t="s">
-        <v>2039</v>
+        <v>2056</v>
       </c>
       <c r="K99" t="s">
-        <v>2040</v>
+        <v>2057</v>
       </c>
       <c r="L99" t="s">
-        <v>2041</v>
+        <v>2058</v>
       </c>
       <c r="M99" t="s">
-        <v>2042</v>
+        <v>2059</v>
       </c>
       <c r="N99" t="s">
-        <v>2043</v>
+        <v>2060</v>
       </c>
       <c r="O99" t="s">
         <v>141</v>
@@ -17511,27 +18381,54 @@
         <v>48</v>
       </c>
       <c r="T99" t="s">
-        <v>2044</v>
+        <v>2061</v>
       </c>
       <c r="U99" t="s">
-        <v>2045</v>
+        <v>2062</v>
       </c>
       <c r="V99" t="s">
-        <v>2046</v>
+        <v>2063</v>
       </c>
       <c r="W99" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X99" t="s">
+        <v>2064</v>
+      </c>
+      <c r="Y99" t="s">
+        <v>2065</v>
+      </c>
+      <c r="Z99" t="s">
+        <v>2066</v>
+      </c>
+      <c r="AA99" t="s">
+        <v>2067</v>
+      </c>
+      <c r="AB99" t="s">
+        <v>2068</v>
+      </c>
+      <c r="AC99" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD99" t="s">
+        <v>2069</v>
+      </c>
+      <c r="AE99" t="s">
+        <v>2070</v>
+      </c>
+      <c r="AF99" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="100" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>2047</v>
+        <v>2071</v>
       </c>
       <c r="B100" t="s">
-        <v>2048</v>
+        <v>2072</v>
       </c>
       <c r="C100" t="s">
-        <v>2049</v>
+        <v>2073</v>
       </c>
       <c r="D100" t="s">
         <v>35</v>
@@ -17545,23 +18442,26 @@
       <c r="G100" t="s">
         <v>203</v>
       </c>
+      <c r="H100" t="s">
+        <v>2074</v>
+      </c>
       <c r="I100" t="s">
-        <v>2050</v>
+        <v>2075</v>
       </c>
       <c r="J100" t="s">
-        <v>2051</v>
+        <v>2076</v>
       </c>
       <c r="K100" t="s">
-        <v>2052</v>
+        <v>2077</v>
       </c>
       <c r="L100" t="s">
-        <v>2053</v>
+        <v>2078</v>
       </c>
       <c r="M100" t="s">
-        <v>2054</v>
+        <v>2079</v>
       </c>
       <c r="N100" t="s">
-        <v>2055</v>
+        <v>2080</v>
       </c>
       <c r="O100" t="s">
         <v>141</v>
@@ -17576,27 +18476,54 @@
         <v>48</v>
       </c>
       <c r="T100" t="s">
-        <v>2056</v>
+        <v>2081</v>
       </c>
       <c r="U100" t="s">
-        <v>2057</v>
+        <v>2082</v>
       </c>
       <c r="V100" t="s">
-        <v>2058</v>
+        <v>2083</v>
       </c>
       <c r="W100" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X100" t="s">
+        <v>2084</v>
+      </c>
+      <c r="Y100" t="s">
+        <v>2085</v>
+      </c>
+      <c r="Z100" t="s">
+        <v>2086</v>
+      </c>
+      <c r="AA100" t="s">
+        <v>2087</v>
+      </c>
+      <c r="AB100" t="s">
+        <v>2088</v>
+      </c>
+      <c r="AC100" t="s">
+        <v>1767</v>
+      </c>
+      <c r="AD100" t="s">
+        <v>2089</v>
+      </c>
+      <c r="AE100" t="s">
+        <v>2090</v>
+      </c>
+      <c r="AF100" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="101" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>2059</v>
+        <v>2091</v>
       </c>
       <c r="B101" t="s">
-        <v>2060</v>
+        <v>2092</v>
       </c>
       <c r="C101" t="s">
-        <v>2061</v>
+        <v>2093</v>
       </c>
       <c r="D101" t="s">
         <v>35</v>
@@ -17610,23 +18537,26 @@
       <c r="G101" t="s">
         <v>89</v>
       </c>
+      <c r="H101" t="s">
+        <v>2094</v>
+      </c>
       <c r="I101" t="s">
-        <v>2062</v>
+        <v>2095</v>
       </c>
       <c r="J101" t="s">
-        <v>2063</v>
+        <v>2096</v>
       </c>
       <c r="K101" t="s">
-        <v>2064</v>
+        <v>2097</v>
       </c>
       <c r="L101" t="s">
-        <v>2065</v>
+        <v>2098</v>
       </c>
       <c r="M101" t="s">
-        <v>2066</v>
+        <v>2099</v>
       </c>
       <c r="N101" t="s">
-        <v>2067</v>
+        <v>2100</v>
       </c>
       <c r="O101" t="s">
         <v>141</v>
@@ -17644,27 +18574,54 @@
         <v>167</v>
       </c>
       <c r="T101" t="s">
-        <v>2068</v>
+        <v>2101</v>
       </c>
       <c r="U101" t="s">
-        <v>2069</v>
+        <v>2102</v>
       </c>
       <c r="V101" t="s">
-        <v>2070</v>
+        <v>2103</v>
       </c>
       <c r="W101" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X101" t="s">
+        <v>2104</v>
+      </c>
+      <c r="Y101" t="s">
+        <v>2105</v>
+      </c>
+      <c r="Z101" t="s">
+        <v>2106</v>
+      </c>
+      <c r="AA101" t="s">
+        <v>2107</v>
+      </c>
+      <c r="AB101" t="s">
+        <v>2108</v>
+      </c>
+      <c r="AC101" t="s">
+        <v>2109</v>
+      </c>
+      <c r="AD101" t="s">
+        <v>2110</v>
+      </c>
+      <c r="AE101" t="s">
+        <v>2111</v>
+      </c>
+      <c r="AF101" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="102" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>2071</v>
+        <v>2112</v>
       </c>
       <c r="B102" t="s">
-        <v>2072</v>
+        <v>2113</v>
       </c>
       <c r="C102" t="s">
-        <v>2073</v>
+        <v>2114</v>
       </c>
       <c r="D102" t="s">
         <v>35</v>
@@ -17678,23 +18635,26 @@
       <c r="G102" t="s">
         <v>203</v>
       </c>
+      <c r="H102" t="s">
+        <v>2115</v>
+      </c>
       <c r="I102" t="s">
-        <v>2074</v>
+        <v>2116</v>
       </c>
       <c r="J102" t="s">
-        <v>2075</v>
+        <v>2117</v>
       </c>
       <c r="K102" t="s">
-        <v>2076</v>
+        <v>2118</v>
       </c>
       <c r="L102" t="s">
-        <v>2077</v>
+        <v>2119</v>
       </c>
       <c r="M102" t="s">
-        <v>2078</v>
+        <v>2120</v>
       </c>
       <c r="N102" t="s">
-        <v>2079</v>
+        <v>2121</v>
       </c>
       <c r="O102" t="s">
         <v>141</v>
@@ -17709,27 +18669,54 @@
         <v>48</v>
       </c>
       <c r="T102" t="s">
-        <v>2080</v>
+        <v>2122</v>
       </c>
       <c r="U102" t="s">
-        <v>2081</v>
+        <v>2123</v>
       </c>
       <c r="V102" t="s">
-        <v>2082</v>
+        <v>2124</v>
       </c>
       <c r="W102" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X102" t="s">
+        <v>2125</v>
+      </c>
+      <c r="Y102" t="s">
+        <v>2126</v>
+      </c>
+      <c r="Z102" t="s">
+        <v>2127</v>
+      </c>
+      <c r="AA102" t="s">
+        <v>2128</v>
+      </c>
+      <c r="AB102" t="s">
+        <v>2129</v>
+      </c>
+      <c r="AC102" t="s">
+        <v>2130</v>
+      </c>
+      <c r="AD102" t="s">
+        <v>2131</v>
+      </c>
+      <c r="AE102" t="s">
+        <v>2132</v>
+      </c>
+      <c r="AF102" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="103" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>2083</v>
+        <v>2133</v>
       </c>
       <c r="B103" t="s">
-        <v>2084</v>
+        <v>2134</v>
       </c>
       <c r="C103" t="s">
-        <v>2085</v>
+        <v>2135</v>
       </c>
       <c r="D103" t="s">
         <v>35</v>
@@ -17743,23 +18730,26 @@
       <c r="G103" t="s">
         <v>203</v>
       </c>
+      <c r="H103" t="s">
+        <v>2136</v>
+      </c>
       <c r="I103" t="s">
-        <v>2086</v>
+        <v>2137</v>
       </c>
       <c r="J103" t="s">
-        <v>2087</v>
+        <v>2138</v>
       </c>
       <c r="K103" t="s">
-        <v>2088</v>
+        <v>2139</v>
       </c>
       <c r="L103" t="s">
-        <v>2089</v>
+        <v>2140</v>
       </c>
       <c r="M103" t="s">
-        <v>2090</v>
+        <v>2141</v>
       </c>
       <c r="N103" t="s">
-        <v>2091</v>
+        <v>2142</v>
       </c>
       <c r="O103" t="s">
         <v>141</v>
@@ -17774,27 +18764,54 @@
         <v>48</v>
       </c>
       <c r="T103" t="s">
-        <v>2092</v>
+        <v>2143</v>
       </c>
       <c r="U103" t="s">
-        <v>2093</v>
+        <v>2144</v>
       </c>
       <c r="V103" t="s">
-        <v>2094</v>
+        <v>2145</v>
       </c>
       <c r="W103" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X103" t="s">
+        <v>2146</v>
+      </c>
+      <c r="Y103" t="s">
+        <v>2147</v>
+      </c>
+      <c r="Z103" t="s">
+        <v>2148</v>
+      </c>
+      <c r="AA103" t="s">
+        <v>2149</v>
+      </c>
+      <c r="AB103" t="s">
+        <v>2150</v>
+      </c>
+      <c r="AC103" t="s">
+        <v>2151</v>
+      </c>
+      <c r="AD103" t="s">
+        <v>2152</v>
+      </c>
+      <c r="AE103" t="s">
+        <v>2153</v>
+      </c>
+      <c r="AF103" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="104" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>2095</v>
+        <v>2154</v>
       </c>
       <c r="B104" t="s">
-        <v>2096</v>
+        <v>2155</v>
       </c>
       <c r="C104" t="s">
-        <v>2097</v>
+        <v>2156</v>
       </c>
       <c r="D104" t="s">
         <v>157</v>
@@ -17808,23 +18825,26 @@
       <c r="G104" t="s">
         <v>158</v>
       </c>
+      <c r="H104" t="s">
+        <v>2157</v>
+      </c>
       <c r="I104" t="s">
-        <v>2098</v>
+        <v>2158</v>
       </c>
       <c r="J104" t="s">
-        <v>2099</v>
+        <v>2159</v>
       </c>
       <c r="K104" t="s">
-        <v>2100</v>
+        <v>2160</v>
       </c>
       <c r="L104" t="s">
-        <v>2101</v>
+        <v>2161</v>
       </c>
       <c r="M104" t="s">
-        <v>2102</v>
+        <v>2162</v>
       </c>
       <c r="N104" t="s">
-        <v>2103</v>
+        <v>2163</v>
       </c>
       <c r="P104" t="s">
         <v>166</v>
@@ -17839,27 +18859,54 @@
         <v>167</v>
       </c>
       <c r="T104" t="s">
-        <v>2104</v>
+        <v>2164</v>
       </c>
       <c r="U104" t="s">
-        <v>2105</v>
+        <v>2165</v>
       </c>
       <c r="V104" t="s">
-        <v>2106</v>
+        <v>2166</v>
       </c>
       <c r="W104" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X104" t="s">
+        <v>2167</v>
+      </c>
+      <c r="Y104" t="s">
+        <v>2168</v>
+      </c>
+      <c r="Z104" t="s">
+        <v>2169</v>
+      </c>
+      <c r="AA104" t="s">
+        <v>2170</v>
+      </c>
+      <c r="AB104" t="s">
+        <v>2171</v>
+      </c>
+      <c r="AC104" t="s">
+        <v>621</v>
+      </c>
+      <c r="AD104" t="s">
+        <v>2172</v>
+      </c>
+      <c r="AE104" t="s">
+        <v>2173</v>
+      </c>
+      <c r="AF104" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="105" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>2107</v>
+        <v>2174</v>
       </c>
       <c r="B105" t="s">
-        <v>2108</v>
+        <v>2175</v>
       </c>
       <c r="C105" t="s">
-        <v>2109</v>
+        <v>2176</v>
       </c>
       <c r="D105" t="s">
         <v>157</v>
@@ -17873,23 +18920,26 @@
       <c r="G105" t="s">
         <v>158</v>
       </c>
+      <c r="H105" t="s">
+        <v>2177</v>
+      </c>
       <c r="I105" t="s">
-        <v>2110</v>
+        <v>2178</v>
       </c>
       <c r="J105" t="s">
-        <v>2111</v>
+        <v>2179</v>
       </c>
       <c r="K105" t="s">
-        <v>2112</v>
+        <v>2180</v>
       </c>
       <c r="L105" t="s">
-        <v>2113</v>
+        <v>2181</v>
       </c>
       <c r="M105" t="s">
-        <v>2114</v>
+        <v>2182</v>
       </c>
       <c r="N105" t="s">
-        <v>2115</v>
+        <v>2183</v>
       </c>
       <c r="P105" t="s">
         <v>166</v>
@@ -17904,27 +18954,54 @@
         <v>167</v>
       </c>
       <c r="T105" t="s">
-        <v>2116</v>
+        <v>2184</v>
       </c>
       <c r="U105" t="s">
-        <v>2117</v>
+        <v>2185</v>
       </c>
       <c r="V105" t="s">
-        <v>2118</v>
+        <v>2186</v>
       </c>
       <c r="W105" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X105" t="s">
+        <v>2187</v>
+      </c>
+      <c r="Y105" t="s">
+        <v>2188</v>
+      </c>
+      <c r="Z105" t="s">
+        <v>2189</v>
+      </c>
+      <c r="AA105" t="s">
+        <v>2190</v>
+      </c>
+      <c r="AB105" t="s">
+        <v>2191</v>
+      </c>
+      <c r="AC105" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD105" t="s">
+        <v>2192</v>
+      </c>
+      <c r="AE105" t="s">
+        <v>2193</v>
+      </c>
+      <c r="AF105" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="106" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>2119</v>
+        <v>2194</v>
       </c>
       <c r="B106" t="s">
-        <v>2120</v>
+        <v>2195</v>
       </c>
       <c r="C106" t="s">
-        <v>2121</v>
+        <v>2196</v>
       </c>
       <c r="D106" t="s">
         <v>65</v>
@@ -17938,23 +19015,26 @@
       <c r="G106" t="s">
         <v>203</v>
       </c>
+      <c r="H106" t="s">
+        <v>2197</v>
+      </c>
       <c r="I106" t="s">
-        <v>2122</v>
+        <v>2198</v>
       </c>
       <c r="J106" t="s">
-        <v>2123</v>
+        <v>2199</v>
       </c>
       <c r="K106" t="s">
-        <v>2124</v>
+        <v>2200</v>
       </c>
       <c r="L106" t="s">
-        <v>2125</v>
+        <v>2201</v>
       </c>
       <c r="M106" t="s">
-        <v>2126</v>
+        <v>2202</v>
       </c>
       <c r="N106" t="s">
-        <v>2127</v>
+        <v>2203</v>
       </c>
       <c r="P106" t="s">
         <v>46</v>
@@ -17966,27 +19046,54 @@
         <v>48</v>
       </c>
       <c r="T106" t="s">
-        <v>2128</v>
+        <v>2204</v>
       </c>
       <c r="U106" t="s">
-        <v>2129</v>
+        <v>2205</v>
       </c>
       <c r="V106" t="s">
-        <v>2130</v>
+        <v>2206</v>
       </c>
       <c r="W106" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X106" t="s">
+        <v>2207</v>
+      </c>
+      <c r="Y106" t="s">
+        <v>2208</v>
+      </c>
+      <c r="Z106" t="s">
+        <v>2209</v>
+      </c>
+      <c r="AA106" t="s">
+        <v>2210</v>
+      </c>
+      <c r="AB106" t="s">
+        <v>2211</v>
+      </c>
+      <c r="AC106" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD106" t="s">
+        <v>2212</v>
+      </c>
+      <c r="AE106" t="s">
+        <v>2213</v>
+      </c>
+      <c r="AF106" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="107" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>2131</v>
+        <v>2214</v>
       </c>
       <c r="B107" t="s">
-        <v>2132</v>
+        <v>2215</v>
       </c>
       <c r="C107" t="s">
-        <v>2133</v>
+        <v>2216</v>
       </c>
       <c r="D107" t="s">
         <v>35</v>
@@ -18000,23 +19107,26 @@
       <c r="G107" t="s">
         <v>158</v>
       </c>
+      <c r="H107" t="s">
+        <v>2217</v>
+      </c>
       <c r="I107" t="s">
-        <v>2134</v>
+        <v>2218</v>
       </c>
       <c r="J107" t="s">
-        <v>2135</v>
+        <v>2219</v>
       </c>
       <c r="K107" t="s">
-        <v>2136</v>
+        <v>2220</v>
       </c>
       <c r="L107" t="s">
-        <v>2137</v>
+        <v>2221</v>
       </c>
       <c r="M107" t="s">
-        <v>2138</v>
+        <v>2222</v>
       </c>
       <c r="N107" t="s">
-        <v>2139</v>
+        <v>2223</v>
       </c>
       <c r="P107" t="s">
         <v>46</v>
@@ -18028,27 +19138,54 @@
         <v>48</v>
       </c>
       <c r="T107" t="s">
-        <v>2140</v>
+        <v>2224</v>
       </c>
       <c r="U107" t="s">
-        <v>2141</v>
+        <v>2225</v>
       </c>
       <c r="V107" t="s">
-        <v>2142</v>
+        <v>2226</v>
       </c>
       <c r="W107" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X107" t="s">
+        <v>2227</v>
+      </c>
+      <c r="Y107" t="s">
+        <v>2228</v>
+      </c>
+      <c r="Z107" t="s">
+        <v>2229</v>
+      </c>
+      <c r="AA107" t="s">
+        <v>2230</v>
+      </c>
+      <c r="AB107" t="s">
+        <v>2231</v>
+      </c>
+      <c r="AC107" t="s">
+        <v>2232</v>
+      </c>
+      <c r="AD107" t="s">
+        <v>2233</v>
+      </c>
+      <c r="AE107" t="s">
+        <v>2234</v>
+      </c>
+      <c r="AF107" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="108" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>2143</v>
+        <v>2235</v>
       </c>
       <c r="B108" t="s">
-        <v>2144</v>
+        <v>2236</v>
       </c>
       <c r="C108" t="s">
-        <v>2145</v>
+        <v>2237</v>
       </c>
       <c r="D108" t="s">
         <v>65</v>
@@ -18062,23 +19199,26 @@
       <c r="G108" t="s">
         <v>331</v>
       </c>
+      <c r="H108" t="s">
+        <v>2238</v>
+      </c>
       <c r="I108" t="s">
-        <v>2146</v>
+        <v>2239</v>
       </c>
       <c r="J108" t="s">
-        <v>2147</v>
+        <v>2240</v>
       </c>
       <c r="K108" t="s">
-        <v>2148</v>
+        <v>2241</v>
       </c>
       <c r="L108" t="s">
-        <v>2149</v>
+        <v>2242</v>
       </c>
       <c r="M108" t="s">
-        <v>2150</v>
+        <v>2243</v>
       </c>
       <c r="N108" t="s">
-        <v>2151</v>
+        <v>2244</v>
       </c>
       <c r="P108" t="s">
         <v>46</v>
@@ -18090,27 +19230,54 @@
         <v>48</v>
       </c>
       <c r="T108" t="s">
-        <v>2152</v>
+        <v>2245</v>
       </c>
       <c r="U108" t="s">
-        <v>2153</v>
+        <v>2246</v>
       </c>
       <c r="V108" t="s">
-        <v>2154</v>
+        <v>2247</v>
       </c>
       <c r="W108" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X108" t="s">
+        <v>2248</v>
+      </c>
+      <c r="Y108" t="s">
+        <v>2249</v>
+      </c>
+      <c r="Z108" t="s">
+        <v>2250</v>
+      </c>
+      <c r="AA108" t="s">
+        <v>2251</v>
+      </c>
+      <c r="AB108" t="s">
+        <v>2252</v>
+      </c>
+      <c r="AC108" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD108" t="s">
+        <v>2253</v>
+      </c>
+      <c r="AE108" t="s">
+        <v>2254</v>
+      </c>
+      <c r="AF108" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="109" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>2155</v>
+        <v>2255</v>
       </c>
       <c r="B109" t="s">
-        <v>2156</v>
+        <v>2256</v>
       </c>
       <c r="C109" t="s">
-        <v>2157</v>
+        <v>2257</v>
       </c>
       <c r="D109" t="s">
         <v>157</v>
@@ -18124,23 +19291,26 @@
       <c r="G109" t="s">
         <v>158</v>
       </c>
+      <c r="H109" t="s">
+        <v>2258</v>
+      </c>
       <c r="I109" t="s">
-        <v>2158</v>
+        <v>2259</v>
       </c>
       <c r="J109" t="s">
-        <v>2159</v>
+        <v>2260</v>
       </c>
       <c r="K109" t="s">
-        <v>2160</v>
+        <v>2261</v>
       </c>
       <c r="L109" t="s">
-        <v>2161</v>
+        <v>2262</v>
       </c>
       <c r="M109" t="s">
-        <v>2162</v>
+        <v>2263</v>
       </c>
       <c r="N109" t="s">
-        <v>2163</v>
+        <v>2264</v>
       </c>
       <c r="P109" t="s">
         <v>166</v>
@@ -18155,27 +19325,54 @@
         <v>167</v>
       </c>
       <c r="T109" t="s">
-        <v>2164</v>
+        <v>2265</v>
       </c>
       <c r="U109" t="s">
-        <v>2165</v>
+        <v>2266</v>
       </c>
       <c r="V109" t="s">
-        <v>2166</v>
+        <v>2267</v>
       </c>
       <c r="W109" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X109" t="s">
+        <v>2268</v>
+      </c>
+      <c r="Y109" t="s">
+        <v>2269</v>
+      </c>
+      <c r="Z109" t="s">
+        <v>2270</v>
+      </c>
+      <c r="AA109" t="s">
+        <v>2271</v>
+      </c>
+      <c r="AB109" t="s">
+        <v>2272</v>
+      </c>
+      <c r="AC109" t="s">
+        <v>621</v>
+      </c>
+      <c r="AD109" t="s">
+        <v>2273</v>
+      </c>
+      <c r="AE109" t="s">
+        <v>2274</v>
+      </c>
+      <c r="AF109" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="110" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>2167</v>
+        <v>2275</v>
       </c>
       <c r="B110" t="s">
-        <v>2168</v>
+        <v>2276</v>
       </c>
       <c r="C110" t="s">
-        <v>2169</v>
+        <v>2277</v>
       </c>
       <c r="D110" t="s">
         <v>157</v>
@@ -18189,23 +19386,26 @@
       <c r="G110" t="s">
         <v>158</v>
       </c>
+      <c r="H110" t="s">
+        <v>2278</v>
+      </c>
       <c r="I110" t="s">
-        <v>2170</v>
+        <v>2279</v>
       </c>
       <c r="J110" t="s">
-        <v>2171</v>
+        <v>2280</v>
       </c>
       <c r="K110" t="s">
-        <v>2172</v>
+        <v>2281</v>
       </c>
       <c r="L110" t="s">
-        <v>2173</v>
+        <v>2282</v>
       </c>
       <c r="M110" t="s">
-        <v>2174</v>
+        <v>2283</v>
       </c>
       <c r="N110" t="s">
-        <v>2175</v>
+        <v>2284</v>
       </c>
       <c r="P110" t="s">
         <v>166</v>
@@ -18220,27 +19420,54 @@
         <v>167</v>
       </c>
       <c r="T110" t="s">
-        <v>2176</v>
+        <v>2285</v>
       </c>
       <c r="U110" t="s">
-        <v>2177</v>
+        <v>2286</v>
       </c>
       <c r="V110" t="s">
-        <v>2178</v>
+        <v>2287</v>
       </c>
       <c r="W110" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X110" t="s">
+        <v>2288</v>
+      </c>
+      <c r="Y110" t="s">
+        <v>2289</v>
+      </c>
+      <c r="Z110" t="s">
+        <v>2290</v>
+      </c>
+      <c r="AA110" t="s">
+        <v>2291</v>
+      </c>
+      <c r="AB110" t="s">
+        <v>2292</v>
+      </c>
+      <c r="AC110" t="s">
+        <v>621</v>
+      </c>
+      <c r="AD110" t="s">
+        <v>2293</v>
+      </c>
+      <c r="AE110" t="s">
+        <v>2294</v>
+      </c>
+      <c r="AF110" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="111" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>2179</v>
+        <v>2295</v>
       </c>
       <c r="B111" t="s">
-        <v>2180</v>
+        <v>2296</v>
       </c>
       <c r="C111" t="s">
-        <v>2181</v>
+        <v>2297</v>
       </c>
       <c r="D111" t="s">
         <v>65</v>
@@ -18254,23 +19481,26 @@
       <c r="G111" t="s">
         <v>89</v>
       </c>
+      <c r="H111" t="s">
+        <v>2298</v>
+      </c>
       <c r="I111" t="s">
-        <v>2182</v>
+        <v>2299</v>
       </c>
       <c r="J111" t="s">
-        <v>2183</v>
+        <v>2300</v>
       </c>
       <c r="K111" t="s">
-        <v>2184</v>
+        <v>2301</v>
       </c>
       <c r="L111" t="s">
-        <v>2185</v>
+        <v>2302</v>
       </c>
       <c r="M111" t="s">
-        <v>2186</v>
+        <v>2303</v>
       </c>
       <c r="N111" t="s">
-        <v>2187</v>
+        <v>2304</v>
       </c>
       <c r="P111" t="s">
         <v>166</v>
@@ -18285,27 +19515,54 @@
         <v>167</v>
       </c>
       <c r="T111" t="s">
-        <v>2188</v>
+        <v>2305</v>
       </c>
       <c r="U111" t="s">
-        <v>2189</v>
+        <v>2306</v>
       </c>
       <c r="V111" t="s">
-        <v>2190</v>
+        <v>2307</v>
       </c>
       <c r="W111" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X111" t="s">
+        <v>2308</v>
+      </c>
+      <c r="Y111" t="s">
+        <v>2309</v>
+      </c>
+      <c r="Z111" t="s">
+        <v>2310</v>
+      </c>
+      <c r="AA111" t="s">
+        <v>2311</v>
+      </c>
+      <c r="AB111" t="s">
+        <v>2312</v>
+      </c>
+      <c r="AC111" t="s">
+        <v>1458</v>
+      </c>
+      <c r="AD111" t="s">
+        <v>2313</v>
+      </c>
+      <c r="AE111" t="s">
+        <v>2314</v>
+      </c>
+      <c r="AF111" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="112" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>2191</v>
+        <v>2315</v>
       </c>
       <c r="B112" t="s">
-        <v>2192</v>
+        <v>2316</v>
       </c>
       <c r="C112" t="s">
-        <v>2193</v>
+        <v>2317</v>
       </c>
       <c r="D112" t="s">
         <v>65</v>
@@ -18319,23 +19576,26 @@
       <c r="G112" t="s">
         <v>203</v>
       </c>
+      <c r="H112" t="s">
+        <v>2318</v>
+      </c>
       <c r="I112" t="s">
-        <v>2194</v>
+        <v>2319</v>
       </c>
       <c r="J112" t="s">
-        <v>2195</v>
+        <v>2320</v>
       </c>
       <c r="K112" t="s">
-        <v>2196</v>
+        <v>2321</v>
       </c>
       <c r="L112" t="s">
-        <v>2197</v>
+        <v>2322</v>
       </c>
       <c r="M112" t="s">
-        <v>2198</v>
+        <v>2323</v>
       </c>
       <c r="N112" t="s">
-        <v>2199</v>
+        <v>2324</v>
       </c>
       <c r="O112" t="s">
         <v>141</v>
@@ -18353,27 +19613,54 @@
         <v>167</v>
       </c>
       <c r="T112" t="s">
-        <v>2200</v>
+        <v>2325</v>
       </c>
       <c r="U112" t="s">
-        <v>2201</v>
+        <v>2326</v>
       </c>
       <c r="V112" t="s">
-        <v>2202</v>
+        <v>2327</v>
       </c>
       <c r="W112" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X112" t="s">
+        <v>2328</v>
+      </c>
+      <c r="Y112" t="s">
+        <v>2329</v>
+      </c>
+      <c r="Z112" t="s">
+        <v>2330</v>
+      </c>
+      <c r="AA112" t="s">
+        <v>2331</v>
+      </c>
+      <c r="AB112" t="s">
+        <v>2332</v>
+      </c>
+      <c r="AC112" t="s">
+        <v>473</v>
+      </c>
+      <c r="AD112" t="s">
+        <v>2333</v>
+      </c>
+      <c r="AE112" t="s">
+        <v>2334</v>
+      </c>
+      <c r="AF112" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="113" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>2203</v>
+        <v>2335</v>
       </c>
       <c r="B113" t="s">
-        <v>2204</v>
+        <v>2336</v>
       </c>
       <c r="C113" t="s">
-        <v>2205</v>
+        <v>2337</v>
       </c>
       <c r="D113" t="s">
         <v>65</v>
@@ -18387,23 +19674,26 @@
       <c r="G113" t="s">
         <v>203</v>
       </c>
+      <c r="H113" t="s">
+        <v>2338</v>
+      </c>
       <c r="I113" t="s">
-        <v>2206</v>
+        <v>2339</v>
       </c>
       <c r="J113" t="s">
-        <v>2207</v>
+        <v>2340</v>
       </c>
       <c r="K113" t="s">
-        <v>2208</v>
+        <v>2341</v>
       </c>
       <c r="L113" t="s">
-        <v>2209</v>
+        <v>2342</v>
       </c>
       <c r="M113" t="s">
-        <v>2210</v>
+        <v>2343</v>
       </c>
       <c r="N113" t="s">
-        <v>2211</v>
+        <v>2344</v>
       </c>
       <c r="O113" t="s">
         <v>141</v>
@@ -18421,27 +19711,54 @@
         <v>167</v>
       </c>
       <c r="T113" t="s">
-        <v>2212</v>
+        <v>2345</v>
       </c>
       <c r="U113" t="s">
-        <v>2213</v>
+        <v>2346</v>
       </c>
       <c r="V113" t="s">
-        <v>2214</v>
+        <v>2347</v>
       </c>
       <c r="W113" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X113" t="s">
+        <v>2348</v>
+      </c>
+      <c r="Y113" t="s">
+        <v>2349</v>
+      </c>
+      <c r="Z113" t="s">
+        <v>2350</v>
+      </c>
+      <c r="AA113" t="s">
+        <v>2351</v>
+      </c>
+      <c r="AB113" t="s">
+        <v>2352</v>
+      </c>
+      <c r="AC113" t="s">
+        <v>683</v>
+      </c>
+      <c r="AD113" t="s">
+        <v>2353</v>
+      </c>
+      <c r="AE113" t="s">
+        <v>2354</v>
+      </c>
+      <c r="AF113" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="114" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>2215</v>
+        <v>2355</v>
       </c>
       <c r="B114" t="s">
-        <v>2216</v>
+        <v>2356</v>
       </c>
       <c r="C114" t="s">
-        <v>2217</v>
+        <v>2357</v>
       </c>
       <c r="D114" t="s">
         <v>35</v>
@@ -18455,23 +19772,26 @@
       <c r="G114" t="s">
         <v>331</v>
       </c>
+      <c r="H114" t="s">
+        <v>2358</v>
+      </c>
       <c r="I114" t="s">
-        <v>2218</v>
+        <v>2359</v>
       </c>
       <c r="J114" t="s">
-        <v>2219</v>
+        <v>2360</v>
       </c>
       <c r="K114" t="s">
-        <v>2220</v>
+        <v>2361</v>
       </c>
       <c r="L114" t="s">
-        <v>2221</v>
+        <v>2362</v>
       </c>
       <c r="M114" t="s">
-        <v>2222</v>
+        <v>2363</v>
       </c>
       <c r="N114" t="s">
-        <v>2223</v>
+        <v>2364</v>
       </c>
       <c r="P114" t="s">
         <v>46</v>
@@ -18483,27 +19803,54 @@
         <v>48</v>
       </c>
       <c r="T114" t="s">
-        <v>2224</v>
+        <v>2365</v>
       </c>
       <c r="U114" t="s">
-        <v>2225</v>
+        <v>2366</v>
       </c>
       <c r="V114" t="s">
-        <v>2226</v>
+        <v>2367</v>
       </c>
       <c r="W114" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X114" t="s">
+        <v>2368</v>
+      </c>
+      <c r="Y114" t="s">
+        <v>2369</v>
+      </c>
+      <c r="Z114" t="s">
+        <v>2370</v>
+      </c>
+      <c r="AA114" t="s">
+        <v>2371</v>
+      </c>
+      <c r="AB114" t="s">
+        <v>2372</v>
+      </c>
+      <c r="AC114" t="s">
+        <v>683</v>
+      </c>
+      <c r="AD114" t="s">
+        <v>2373</v>
+      </c>
+      <c r="AE114" t="s">
+        <v>2374</v>
+      </c>
+      <c r="AF114" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="115" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>2227</v>
+        <v>2375</v>
       </c>
       <c r="B115" t="s">
-        <v>2228</v>
+        <v>2376</v>
       </c>
       <c r="C115" t="s">
-        <v>2229</v>
+        <v>2377</v>
       </c>
       <c r="D115" t="s">
         <v>65</v>
@@ -18517,23 +19864,26 @@
       <c r="G115" t="s">
         <v>331</v>
       </c>
+      <c r="H115" t="s">
+        <v>2378</v>
+      </c>
       <c r="I115" t="s">
-        <v>2230</v>
+        <v>2379</v>
       </c>
       <c r="J115" t="s">
-        <v>2231</v>
+        <v>2380</v>
       </c>
       <c r="K115" t="s">
-        <v>2232</v>
+        <v>2381</v>
       </c>
       <c r="L115" t="s">
-        <v>2233</v>
+        <v>2382</v>
       </c>
       <c r="M115" t="s">
-        <v>2234</v>
+        <v>2383</v>
       </c>
       <c r="N115" t="s">
-        <v>2235</v>
+        <v>2384</v>
       </c>
       <c r="P115" t="s">
         <v>46</v>
@@ -18545,27 +19895,54 @@
         <v>48</v>
       </c>
       <c r="T115" t="s">
-        <v>2236</v>
+        <v>2385</v>
       </c>
       <c r="U115" t="s">
-        <v>2237</v>
+        <v>2386</v>
       </c>
       <c r="V115" t="s">
-        <v>2238</v>
+        <v>2387</v>
       </c>
       <c r="W115" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X115" t="s">
+        <v>2388</v>
+      </c>
+      <c r="Y115" t="s">
+        <v>2389</v>
+      </c>
+      <c r="Z115" t="s">
+        <v>2390</v>
+      </c>
+      <c r="AA115" t="s">
+        <v>2391</v>
+      </c>
+      <c r="AB115" t="s">
+        <v>2392</v>
+      </c>
+      <c r="AC115" t="s">
+        <v>473</v>
+      </c>
+      <c r="AD115" t="s">
+        <v>2393</v>
+      </c>
+      <c r="AE115" t="s">
+        <v>2394</v>
+      </c>
+      <c r="AF115" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="116" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>2239</v>
+        <v>2395</v>
       </c>
       <c r="B116" t="s">
-        <v>2240</v>
+        <v>2396</v>
       </c>
       <c r="C116" t="s">
-        <v>2241</v>
+        <v>2397</v>
       </c>
       <c r="D116" t="s">
         <v>65</v>
@@ -18579,23 +19956,26 @@
       <c r="G116" t="s">
         <v>203</v>
       </c>
+      <c r="H116" t="s">
+        <v>2398</v>
+      </c>
       <c r="I116" t="s">
-        <v>2242</v>
+        <v>2399</v>
       </c>
       <c r="J116" t="s">
-        <v>2243</v>
+        <v>2400</v>
       </c>
       <c r="K116" t="s">
-        <v>2244</v>
+        <v>2401</v>
       </c>
       <c r="L116" t="s">
-        <v>2245</v>
+        <v>2402</v>
       </c>
       <c r="M116" t="s">
-        <v>2246</v>
+        <v>2403</v>
       </c>
       <c r="N116" t="s">
-        <v>2247</v>
+        <v>2404</v>
       </c>
       <c r="P116" t="s">
         <v>46</v>
@@ -18607,27 +19987,54 @@
         <v>48</v>
       </c>
       <c r="T116" t="s">
-        <v>2248</v>
+        <v>2405</v>
       </c>
       <c r="U116" t="s">
-        <v>2249</v>
+        <v>2406</v>
       </c>
       <c r="V116" t="s">
-        <v>2250</v>
+        <v>2407</v>
       </c>
       <c r="W116" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X116" t="s">
+        <v>2408</v>
+      </c>
+      <c r="Y116" t="s">
+        <v>2409</v>
+      </c>
+      <c r="Z116" t="s">
+        <v>2410</v>
+      </c>
+      <c r="AA116" t="s">
+        <v>2411</v>
+      </c>
+      <c r="AB116" t="s">
+        <v>2412</v>
+      </c>
+      <c r="AC116" t="s">
+        <v>1788</v>
+      </c>
+      <c r="AD116" t="s">
+        <v>2413</v>
+      </c>
+      <c r="AE116" t="s">
+        <v>2414</v>
+      </c>
+      <c r="AF116" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="117" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>2251</v>
+        <v>2415</v>
       </c>
       <c r="B117" t="s">
-        <v>2252</v>
+        <v>2416</v>
       </c>
       <c r="C117" t="s">
-        <v>2253</v>
+        <v>2417</v>
       </c>
       <c r="D117" t="s">
         <v>35</v>
@@ -18641,23 +20048,26 @@
       <c r="G117" t="s">
         <v>331</v>
       </c>
+      <c r="H117" t="s">
+        <v>2418</v>
+      </c>
       <c r="I117" t="s">
-        <v>2254</v>
+        <v>2419</v>
       </c>
       <c r="J117" t="s">
-        <v>2255</v>
+        <v>2420</v>
       </c>
       <c r="K117" t="s">
-        <v>2256</v>
+        <v>2421</v>
       </c>
       <c r="L117" t="s">
-        <v>2257</v>
+        <v>2422</v>
       </c>
       <c r="M117" t="s">
-        <v>2258</v>
+        <v>2423</v>
       </c>
       <c r="N117" t="s">
-        <v>2259</v>
+        <v>2424</v>
       </c>
       <c r="O117" t="s">
         <v>141</v>
@@ -18675,27 +20085,54 @@
         <v>167</v>
       </c>
       <c r="T117" t="s">
-        <v>2260</v>
+        <v>2425</v>
       </c>
       <c r="U117" t="s">
-        <v>2261</v>
+        <v>2426</v>
       </c>
       <c r="V117" t="s">
-        <v>2262</v>
+        <v>2427</v>
       </c>
       <c r="W117" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X117" t="s">
+        <v>2428</v>
+      </c>
+      <c r="Y117" t="s">
+        <v>2429</v>
+      </c>
+      <c r="Z117" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AA117" t="s">
+        <v>2431</v>
+      </c>
+      <c r="AB117" t="s">
+        <v>2432</v>
+      </c>
+      <c r="AC117" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD117" t="s">
+        <v>2433</v>
+      </c>
+      <c r="AE117" t="s">
+        <v>2434</v>
+      </c>
+      <c r="AF117" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="118" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>2263</v>
+        <v>2435</v>
       </c>
       <c r="B118" t="s">
-        <v>2264</v>
+        <v>2436</v>
       </c>
       <c r="C118" t="s">
-        <v>2265</v>
+        <v>2437</v>
       </c>
       <c r="D118" t="s">
         <v>157</v>
@@ -18709,23 +20146,26 @@
       <c r="G118" t="s">
         <v>158</v>
       </c>
+      <c r="H118" t="s">
+        <v>2438</v>
+      </c>
       <c r="I118" t="s">
-        <v>2266</v>
+        <v>2439</v>
       </c>
       <c r="J118" t="s">
-        <v>2267</v>
+        <v>2440</v>
       </c>
       <c r="K118" t="s">
-        <v>2268</v>
+        <v>2441</v>
       </c>
       <c r="L118" t="s">
-        <v>2269</v>
+        <v>2442</v>
       </c>
       <c r="M118" t="s">
-        <v>2270</v>
+        <v>2443</v>
       </c>
       <c r="N118" t="s">
-        <v>2271</v>
+        <v>2444</v>
       </c>
       <c r="P118" t="s">
         <v>166</v>
@@ -18740,27 +20180,54 @@
         <v>167</v>
       </c>
       <c r="T118" t="s">
-        <v>2272</v>
+        <v>2445</v>
       </c>
       <c r="U118" t="s">
-        <v>2273</v>
+        <v>2446</v>
       </c>
       <c r="V118" t="s">
-        <v>2274</v>
+        <v>2447</v>
       </c>
       <c r="W118" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X118" t="s">
+        <v>2448</v>
+      </c>
+      <c r="Y118" t="s">
+        <v>2449</v>
+      </c>
+      <c r="Z118" t="s">
+        <v>2450</v>
+      </c>
+      <c r="AA118" t="s">
+        <v>2451</v>
+      </c>
+      <c r="AB118" t="s">
+        <v>2452</v>
+      </c>
+      <c r="AC118" t="s">
+        <v>621</v>
+      </c>
+      <c r="AD118" t="s">
+        <v>2453</v>
+      </c>
+      <c r="AE118" t="s">
+        <v>2454</v>
+      </c>
+      <c r="AF118" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="119" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>2275</v>
+        <v>2455</v>
       </c>
       <c r="B119" t="s">
-        <v>2276</v>
+        <v>2456</v>
       </c>
       <c r="C119" t="s">
-        <v>2277</v>
+        <v>2457</v>
       </c>
       <c r="D119" t="s">
         <v>35</v>
@@ -18774,23 +20241,26 @@
       <c r="G119" t="s">
         <v>203</v>
       </c>
+      <c r="H119" t="s">
+        <v>2458</v>
+      </c>
       <c r="I119" t="s">
-        <v>2278</v>
+        <v>2459</v>
       </c>
       <c r="J119" t="s">
-        <v>2279</v>
+        <v>2460</v>
       </c>
       <c r="K119" t="s">
-        <v>2280</v>
+        <v>2461</v>
       </c>
       <c r="L119" t="s">
-        <v>2281</v>
+        <v>2462</v>
       </c>
       <c r="M119" t="s">
-        <v>2282</v>
+        <v>2463</v>
       </c>
       <c r="N119" t="s">
-        <v>2283</v>
+        <v>2464</v>
       </c>
       <c r="O119" t="s">
         <v>141</v>
@@ -18805,27 +20275,54 @@
         <v>48</v>
       </c>
       <c r="T119" t="s">
-        <v>2284</v>
+        <v>2465</v>
       </c>
       <c r="U119" t="s">
-        <v>2285</v>
+        <v>2466</v>
       </c>
       <c r="V119" t="s">
-        <v>2286</v>
+        <v>2467</v>
       </c>
       <c r="W119" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X119" t="s">
+        <v>2468</v>
+      </c>
+      <c r="Y119" t="s">
+        <v>2469</v>
+      </c>
+      <c r="Z119" t="s">
+        <v>2470</v>
+      </c>
+      <c r="AA119" t="s">
+        <v>2471</v>
+      </c>
+      <c r="AB119" t="s">
+        <v>2472</v>
+      </c>
+      <c r="AC119" t="s">
+        <v>1788</v>
+      </c>
+      <c r="AD119" t="s">
+        <v>2473</v>
+      </c>
+      <c r="AE119" t="s">
+        <v>2474</v>
+      </c>
+      <c r="AF119" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="120" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>2287</v>
+        <v>2475</v>
       </c>
       <c r="B120" t="s">
-        <v>2288</v>
+        <v>2476</v>
       </c>
       <c r="C120" t="s">
-        <v>2289</v>
+        <v>2477</v>
       </c>
       <c r="D120" t="s">
         <v>65</v>
@@ -18839,23 +20336,26 @@
       <c r="G120" t="s">
         <v>203</v>
       </c>
+      <c r="H120" t="s">
+        <v>2478</v>
+      </c>
       <c r="I120" t="s">
-        <v>2290</v>
+        <v>2479</v>
       </c>
       <c r="J120" t="s">
-        <v>2291</v>
+        <v>2480</v>
       </c>
       <c r="K120" t="s">
-        <v>2292</v>
+        <v>2481</v>
       </c>
       <c r="L120" t="s">
-        <v>2293</v>
+        <v>2482</v>
       </c>
       <c r="M120" t="s">
-        <v>2294</v>
+        <v>2483</v>
       </c>
       <c r="N120" t="s">
-        <v>2295</v>
+        <v>2484</v>
       </c>
       <c r="P120" t="s">
         <v>46</v>
@@ -18867,27 +20367,54 @@
         <v>48</v>
       </c>
       <c r="T120" t="s">
-        <v>2296</v>
+        <v>2485</v>
       </c>
       <c r="U120" t="s">
-        <v>2297</v>
+        <v>2486</v>
       </c>
       <c r="V120" t="s">
-        <v>2298</v>
+        <v>2487</v>
       </c>
       <c r="W120" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X120" t="s">
+        <v>2488</v>
+      </c>
+      <c r="Y120" t="s">
+        <v>2489</v>
+      </c>
+      <c r="Z120" t="s">
+        <v>2490</v>
+      </c>
+      <c r="AA120" t="s">
+        <v>2491</v>
+      </c>
+      <c r="AB120" t="s">
+        <v>2492</v>
+      </c>
+      <c r="AC120" t="s">
+        <v>683</v>
+      </c>
+      <c r="AD120" t="s">
+        <v>2493</v>
+      </c>
+      <c r="AE120" t="s">
+        <v>2494</v>
+      </c>
+      <c r="AF120" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="121" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>2299</v>
+        <v>2495</v>
       </c>
       <c r="B121" t="s">
-        <v>2300</v>
+        <v>2496</v>
       </c>
       <c r="C121" t="s">
-        <v>2301</v>
+        <v>2497</v>
       </c>
       <c r="D121" t="s">
         <v>35</v>
@@ -18901,23 +20428,26 @@
       <c r="G121" t="s">
         <v>89</v>
       </c>
+      <c r="H121" t="s">
+        <v>2498</v>
+      </c>
       <c r="I121" t="s">
-        <v>2302</v>
+        <v>2499</v>
       </c>
       <c r="J121" t="s">
-        <v>2303</v>
+        <v>2500</v>
       </c>
       <c r="K121" t="s">
-        <v>2304</v>
+        <v>2501</v>
       </c>
       <c r="L121" t="s">
-        <v>2305</v>
+        <v>2502</v>
       </c>
       <c r="M121" t="s">
-        <v>2306</v>
+        <v>2503</v>
       </c>
       <c r="N121" t="s">
-        <v>2307</v>
+        <v>2504</v>
       </c>
       <c r="O121" t="s">
         <v>141</v>
@@ -18932,27 +20462,54 @@
         <v>48</v>
       </c>
       <c r="T121" t="s">
-        <v>2308</v>
+        <v>2505</v>
       </c>
       <c r="U121" t="s">
-        <v>2309</v>
+        <v>2506</v>
       </c>
       <c r="V121" t="s">
-        <v>2310</v>
+        <v>2507</v>
       </c>
       <c r="W121" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X121" t="s">
+        <v>2508</v>
+      </c>
+      <c r="Y121" t="s">
+        <v>2509</v>
+      </c>
+      <c r="Z121" t="s">
+        <v>2510</v>
+      </c>
+      <c r="AA121" t="s">
+        <v>2511</v>
+      </c>
+      <c r="AB121" t="s">
+        <v>2512</v>
+      </c>
+      <c r="AC121" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD121" t="s">
+        <v>2513</v>
+      </c>
+      <c r="AE121" t="s">
+        <v>2514</v>
+      </c>
+      <c r="AF121" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="122" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>2311</v>
+        <v>2515</v>
       </c>
       <c r="B122" t="s">
-        <v>2312</v>
+        <v>2516</v>
       </c>
       <c r="C122" t="s">
-        <v>2313</v>
+        <v>2517</v>
       </c>
       <c r="D122" t="s">
         <v>65</v>
@@ -18966,23 +20523,26 @@
       <c r="G122" t="s">
         <v>331</v>
       </c>
+      <c r="H122" t="s">
+        <v>2518</v>
+      </c>
       <c r="I122" t="s">
-        <v>2314</v>
+        <v>2519</v>
       </c>
       <c r="J122" t="s">
-        <v>2315</v>
+        <v>2520</v>
       </c>
       <c r="K122" t="s">
-        <v>2316</v>
+        <v>2521</v>
       </c>
       <c r="L122" t="s">
-        <v>2317</v>
+        <v>2522</v>
       </c>
       <c r="M122" t="s">
-        <v>2318</v>
+        <v>2523</v>
       </c>
       <c r="N122" t="s">
-        <v>2319</v>
+        <v>2524</v>
       </c>
       <c r="P122" t="s">
         <v>46</v>
@@ -18994,27 +20554,54 @@
         <v>48</v>
       </c>
       <c r="T122" t="s">
-        <v>2320</v>
+        <v>2525</v>
       </c>
       <c r="U122" t="s">
-        <v>2321</v>
+        <v>2526</v>
       </c>
       <c r="V122" t="s">
-        <v>2322</v>
+        <v>2527</v>
       </c>
       <c r="W122" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X122" t="s">
+        <v>2528</v>
+      </c>
+      <c r="Y122" t="s">
+        <v>2529</v>
+      </c>
+      <c r="Z122" t="s">
+        <v>2530</v>
+      </c>
+      <c r="AA122" t="s">
+        <v>2531</v>
+      </c>
+      <c r="AB122" t="s">
+        <v>2532</v>
+      </c>
+      <c r="AC122" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD122" t="s">
+        <v>2533</v>
+      </c>
+      <c r="AE122" t="s">
+        <v>2534</v>
+      </c>
+      <c r="AF122" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="123" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>2323</v>
+        <v>2535</v>
       </c>
       <c r="B123" t="s">
-        <v>2324</v>
+        <v>2536</v>
       </c>
       <c r="C123" t="s">
-        <v>2325</v>
+        <v>2537</v>
       </c>
       <c r="D123" t="s">
         <v>65</v>
@@ -19028,23 +20615,26 @@
       <c r="G123" t="s">
         <v>203</v>
       </c>
+      <c r="H123" t="s">
+        <v>2538</v>
+      </c>
       <c r="I123" t="s">
-        <v>2326</v>
+        <v>2539</v>
       </c>
       <c r="J123" t="s">
-        <v>2327</v>
+        <v>2540</v>
       </c>
       <c r="K123" t="s">
-        <v>2328</v>
+        <v>2541</v>
       </c>
       <c r="L123" t="s">
-        <v>2329</v>
+        <v>2542</v>
       </c>
       <c r="M123" t="s">
-        <v>2330</v>
+        <v>2543</v>
       </c>
       <c r="N123" t="s">
-        <v>2331</v>
+        <v>2544</v>
       </c>
       <c r="P123" t="s">
         <v>46</v>
@@ -19056,27 +20646,54 @@
         <v>48</v>
       </c>
       <c r="T123" t="s">
-        <v>2332</v>
+        <v>2545</v>
       </c>
       <c r="U123" t="s">
-        <v>2333</v>
+        <v>2546</v>
       </c>
       <c r="V123" t="s">
-        <v>2334</v>
+        <v>2547</v>
       </c>
       <c r="W123" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X123" t="s">
+        <v>2548</v>
+      </c>
+      <c r="Y123" t="s">
+        <v>2549</v>
+      </c>
+      <c r="Z123" t="s">
+        <v>2550</v>
+      </c>
+      <c r="AA123" t="s">
+        <v>2551</v>
+      </c>
+      <c r="AB123" t="s">
+        <v>2552</v>
+      </c>
+      <c r="AC123" t="s">
+        <v>2130</v>
+      </c>
+      <c r="AD123" t="s">
+        <v>2553</v>
+      </c>
+      <c r="AE123" t="s">
+        <v>2554</v>
+      </c>
+      <c r="AF123" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="124" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>2335</v>
+        <v>2555</v>
       </c>
       <c r="B124" t="s">
-        <v>2336</v>
+        <v>2556</v>
       </c>
       <c r="C124" t="s">
-        <v>2337</v>
+        <v>2557</v>
       </c>
       <c r="D124" t="s">
         <v>65</v>
@@ -19090,23 +20707,26 @@
       <c r="G124" t="s">
         <v>331</v>
       </c>
+      <c r="H124" t="s">
+        <v>2558</v>
+      </c>
       <c r="I124" t="s">
-        <v>2338</v>
+        <v>2559</v>
       </c>
       <c r="J124" t="s">
-        <v>2339</v>
+        <v>2560</v>
       </c>
       <c r="K124" t="s">
-        <v>2340</v>
+        <v>2561</v>
       </c>
       <c r="L124" t="s">
-        <v>2341</v>
+        <v>2562</v>
       </c>
       <c r="M124" t="s">
-        <v>2342</v>
+        <v>2563</v>
       </c>
       <c r="N124" t="s">
-        <v>2343</v>
+        <v>2564</v>
       </c>
       <c r="P124" t="s">
         <v>46</v>
@@ -19118,27 +20738,54 @@
         <v>48</v>
       </c>
       <c r="T124" t="s">
-        <v>2344</v>
+        <v>2565</v>
       </c>
       <c r="U124" t="s">
-        <v>2345</v>
+        <v>2566</v>
       </c>
       <c r="V124" t="s">
-        <v>2346</v>
+        <v>2567</v>
       </c>
       <c r="W124" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X124" t="s">
+        <v>2568</v>
+      </c>
+      <c r="Y124" t="s">
+        <v>2569</v>
+      </c>
+      <c r="Z124" t="s">
+        <v>2570</v>
+      </c>
+      <c r="AA124" t="s">
+        <v>2571</v>
+      </c>
+      <c r="AB124" t="s">
+        <v>2572</v>
+      </c>
+      <c r="AC124" t="s">
+        <v>683</v>
+      </c>
+      <c r="AD124" t="s">
+        <v>2573</v>
+      </c>
+      <c r="AE124" t="s">
+        <v>2574</v>
+      </c>
+      <c r="AF124" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="125" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>2347</v>
+        <v>2575</v>
       </c>
       <c r="B125" t="s">
-        <v>2348</v>
+        <v>2576</v>
       </c>
       <c r="C125" t="s">
-        <v>2349</v>
+        <v>2577</v>
       </c>
       <c r="D125" t="s">
         <v>35</v>
@@ -19152,23 +20799,26 @@
       <c r="G125" t="s">
         <v>203</v>
       </c>
+      <c r="H125" t="s">
+        <v>2578</v>
+      </c>
       <c r="I125" t="s">
-        <v>2350</v>
+        <v>2579</v>
       </c>
       <c r="J125" t="s">
-        <v>2351</v>
+        <v>2580</v>
       </c>
       <c r="K125" t="s">
-        <v>2352</v>
+        <v>2581</v>
       </c>
       <c r="L125" t="s">
-        <v>2353</v>
+        <v>2582</v>
       </c>
       <c r="M125" t="s">
-        <v>2354</v>
+        <v>2583</v>
       </c>
       <c r="N125" t="s">
-        <v>2355</v>
+        <v>2584</v>
       </c>
       <c r="O125" t="s">
         <v>141</v>
@@ -19183,27 +20833,54 @@
         <v>48</v>
       </c>
       <c r="T125" t="s">
-        <v>2356</v>
+        <v>2585</v>
       </c>
       <c r="U125" t="s">
-        <v>2357</v>
+        <v>2586</v>
       </c>
       <c r="V125" t="s">
-        <v>2358</v>
+        <v>2587</v>
       </c>
       <c r="W125" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X125" t="s">
+        <v>2588</v>
+      </c>
+      <c r="Y125" t="s">
+        <v>2589</v>
+      </c>
+      <c r="Z125" t="s">
+        <v>2590</v>
+      </c>
+      <c r="AA125" t="s">
+        <v>2591</v>
+      </c>
+      <c r="AB125" t="s">
+        <v>2592</v>
+      </c>
+      <c r="AC125" t="s">
+        <v>1746</v>
+      </c>
+      <c r="AD125" t="s">
+        <v>2593</v>
+      </c>
+      <c r="AE125" t="s">
+        <v>2594</v>
+      </c>
+      <c r="AF125" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="126" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>2359</v>
+        <v>2595</v>
       </c>
       <c r="B126" t="s">
-        <v>2360</v>
+        <v>2596</v>
       </c>
       <c r="C126" t="s">
-        <v>2361</v>
+        <v>2597</v>
       </c>
       <c r="D126" t="s">
         <v>65</v>
@@ -19217,23 +20894,26 @@
       <c r="G126" t="s">
         <v>38</v>
       </c>
+      <c r="H126" t="s">
+        <v>2598</v>
+      </c>
       <c r="I126" t="s">
-        <v>2362</v>
+        <v>2599</v>
       </c>
       <c r="J126" t="s">
-        <v>2363</v>
+        <v>2600</v>
       </c>
       <c r="K126" t="s">
-        <v>2364</v>
+        <v>2601</v>
       </c>
       <c r="L126" t="s">
-        <v>2365</v>
+        <v>2602</v>
       </c>
       <c r="M126" t="s">
-        <v>2366</v>
+        <v>2603</v>
       </c>
       <c r="N126" t="s">
-        <v>2367</v>
+        <v>2604</v>
       </c>
       <c r="O126" t="s">
         <v>141</v>
@@ -19251,27 +20931,54 @@
         <v>167</v>
       </c>
       <c r="T126" t="s">
-        <v>2368</v>
+        <v>2605</v>
       </c>
       <c r="U126" t="s">
-        <v>2369</v>
+        <v>2606</v>
       </c>
       <c r="V126" t="s">
-        <v>2370</v>
+        <v>2607</v>
       </c>
       <c r="W126" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X126" t="s">
+        <v>2608</v>
+      </c>
+      <c r="Y126" t="s">
+        <v>2609</v>
+      </c>
+      <c r="Z126" t="s">
+        <v>2610</v>
+      </c>
+      <c r="AA126" t="s">
+        <v>2611</v>
+      </c>
+      <c r="AB126" t="s">
+        <v>2612</v>
+      </c>
+      <c r="AC126" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD126" t="s">
+        <v>2613</v>
+      </c>
+      <c r="AE126" t="s">
+        <v>2614</v>
+      </c>
+      <c r="AF126" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="127" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>2371</v>
+        <v>2615</v>
       </c>
       <c r="B127" t="s">
-        <v>2372</v>
+        <v>2616</v>
       </c>
       <c r="C127" t="s">
-        <v>2373</v>
+        <v>2617</v>
       </c>
       <c r="D127" t="s">
         <v>157</v>
@@ -19285,20 +20992,23 @@
       <c r="G127" t="s">
         <v>158</v>
       </c>
+      <c r="H127" t="s">
+        <v>2618</v>
+      </c>
       <c r="I127" t="s">
-        <v>2374</v>
+        <v>2619</v>
       </c>
       <c r="J127" t="s">
-        <v>2375</v>
+        <v>2620</v>
       </c>
       <c r="K127" t="s">
-        <v>2376</v>
+        <v>2621</v>
       </c>
       <c r="M127" t="s">
-        <v>2377</v>
+        <v>2622</v>
       </c>
       <c r="N127" t="s">
-        <v>2378</v>
+        <v>2623</v>
       </c>
       <c r="O127" t="s">
         <v>141</v>
@@ -19316,27 +21026,54 @@
         <v>1534</v>
       </c>
       <c r="T127" t="s">
-        <v>2379</v>
+        <v>2624</v>
       </c>
       <c r="U127" t="s">
-        <v>2380</v>
+        <v>2625</v>
       </c>
       <c r="V127" t="s">
-        <v>2381</v>
+        <v>2626</v>
       </c>
       <c r="W127" s="1" t="s">
         <v>1538</v>
+      </c>
+      <c r="X127" t="s">
+        <v>2627</v>
+      </c>
+      <c r="Y127" t="s">
+        <v>2628</v>
+      </c>
+      <c r="Z127" t="s">
+        <v>2629</v>
+      </c>
+      <c r="AA127" t="s">
+        <v>2630</v>
+      </c>
+      <c r="AB127" t="s">
+        <v>2631</v>
+      </c>
+      <c r="AC127" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD127" t="s">
+        <v>2632</v>
+      </c>
+      <c r="AE127" t="s">
+        <v>2633</v>
+      </c>
+      <c r="AF127" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="128" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>2382</v>
+        <v>2634</v>
       </c>
       <c r="B128" t="s">
-        <v>2383</v>
+        <v>2635</v>
       </c>
       <c r="C128" t="s">
-        <v>2384</v>
+        <v>2636</v>
       </c>
       <c r="D128" t="s">
         <v>65</v>
@@ -19350,23 +21087,26 @@
       <c r="G128" t="s">
         <v>203</v>
       </c>
+      <c r="H128" t="s">
+        <v>2637</v>
+      </c>
       <c r="I128" t="s">
-        <v>2385</v>
+        <v>2638</v>
       </c>
       <c r="J128" t="s">
-        <v>2386</v>
+        <v>2639</v>
       </c>
       <c r="K128" t="s">
-        <v>2387</v>
+        <v>2640</v>
       </c>
       <c r="L128" t="s">
-        <v>2388</v>
+        <v>2641</v>
       </c>
       <c r="M128" t="s">
-        <v>2389</v>
+        <v>2642</v>
       </c>
       <c r="N128" t="s">
-        <v>2390</v>
+        <v>2643</v>
       </c>
       <c r="P128" t="s">
         <v>46</v>
@@ -19378,27 +21118,54 @@
         <v>48</v>
       </c>
       <c r="T128" t="s">
-        <v>2391</v>
+        <v>2644</v>
       </c>
       <c r="U128" t="s">
-        <v>2392</v>
+        <v>2645</v>
       </c>
       <c r="V128" t="s">
-        <v>2393</v>
+        <v>2646</v>
       </c>
       <c r="W128" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X128" t="s">
+        <v>2647</v>
+      </c>
+      <c r="Y128" t="s">
+        <v>2648</v>
+      </c>
+      <c r="Z128" t="s">
+        <v>2649</v>
+      </c>
+      <c r="AA128" t="s">
+        <v>2650</v>
+      </c>
+      <c r="AB128" t="s">
+        <v>2651</v>
+      </c>
+      <c r="AC128" t="s">
+        <v>2652</v>
+      </c>
+      <c r="AD128" t="s">
+        <v>2653</v>
+      </c>
+      <c r="AE128" t="s">
+        <v>2654</v>
+      </c>
+      <c r="AF128" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="129" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>2394</v>
+        <v>2655</v>
       </c>
       <c r="B129" t="s">
-        <v>2395</v>
+        <v>2656</v>
       </c>
       <c r="C129" t="s">
-        <v>2396</v>
+        <v>2657</v>
       </c>
       <c r="D129" t="s">
         <v>35</v>
@@ -19412,23 +21179,26 @@
       <c r="G129" t="s">
         <v>203</v>
       </c>
+      <c r="H129" t="s">
+        <v>2658</v>
+      </c>
       <c r="I129" t="s">
-        <v>2397</v>
+        <v>2659</v>
       </c>
       <c r="J129" t="s">
-        <v>2398</v>
+        <v>2660</v>
       </c>
       <c r="K129" t="s">
-        <v>2399</v>
+        <v>2661</v>
       </c>
       <c r="L129" t="s">
-        <v>2400</v>
+        <v>2662</v>
       </c>
       <c r="M129" t="s">
-        <v>2401</v>
+        <v>2663</v>
       </c>
       <c r="N129" t="s">
-        <v>2402</v>
+        <v>2664</v>
       </c>
       <c r="P129" t="s">
         <v>46</v>
@@ -19440,16 +21210,43 @@
         <v>48</v>
       </c>
       <c r="T129" t="s">
-        <v>2403</v>
+        <v>2665</v>
       </c>
       <c r="U129" t="s">
-        <v>2404</v>
+        <v>2666</v>
       </c>
       <c r="V129" t="s">
-        <v>2405</v>
+        <v>2667</v>
       </c>
       <c r="W129" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="X129" t="s">
+        <v>2668</v>
+      </c>
+      <c r="Y129" t="s">
+        <v>2669</v>
+      </c>
+      <c r="Z129" t="s">
+        <v>2670</v>
+      </c>
+      <c r="AA129" t="s">
+        <v>2671</v>
+      </c>
+      <c r="AB129" t="s">
+        <v>2672</v>
+      </c>
+      <c r="AC129" t="s">
+        <v>787</v>
+      </c>
+      <c r="AD129" t="s">
+        <v>2673</v>
+      </c>
+      <c r="AE129" t="s">
+        <v>2674</v>
+      </c>
+      <c r="AF129" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>